<commit_message>
added the analysis sheet.
</commit_message>
<xml_diff>
--- a/Personal Budget - English.xlsx
+++ b/Personal Budget - English.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rcssi\Code\Personal_Finance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45F7FAEE-E712-4CA9-BA89-B28959D6A5D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7C8CCEE-EBEA-4CDA-AF34-F623BC86246C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-114" yWindow="-114" windowWidth="19704" windowHeight="11178" tabRatio="792" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,8 @@
     <sheet name="Balance &amp; Tracking" sheetId="12" r:id="rId2"/>
     <sheet name="Net Salary" sheetId="8" state="hidden" r:id="rId3"/>
     <sheet name="Expenses" sheetId="1" state="hidden" r:id="rId4"/>
-    <sheet name="Dashbord" sheetId="13" r:id="rId5"/>
+    <sheet name="Analysis" sheetId="16" state="hidden" r:id="rId5"/>
+    <sheet name="Dashbord" sheetId="13" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="Accounts">'Data Validation'!$B$5:$B$9</definedName>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -75,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="87">
   <si>
     <t>Total</t>
   </si>
@@ -317,18 +318,37 @@
     <t>Initial Balance</t>
   </si>
   <si>
-    <t>Info</t>
+    <t>TAB' to create a new line.</t>
+  </si>
+  <si>
+    <t>Totol</t>
+  </si>
+  <si>
+    <t>Próximo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Select - </t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Interval</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="mmmm"/>
     <numFmt numFmtId="165" formatCode="dd/mm"/>
     <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    <numFmt numFmtId="167" formatCode="dd/mmmm"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -601,7 +621,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -770,9 +790,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="166" fontId="4" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -787,7 +804,33 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -7427,7 +7470,7 @@
       <c r="B5" s="70" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="77">
+      <c r="C5" s="76">
         <v>0</v>
       </c>
       <c r="E5" s="70" t="s">
@@ -7455,7 +7498,7 @@
       <c r="B6" s="70" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="77">
+      <c r="C6" s="76">
         <v>0</v>
       </c>
       <c r="E6" s="70" t="s">
@@ -7481,7 +7524,7 @@
       <c r="B7" s="70" t="s">
         <v>77</v>
       </c>
-      <c r="C7" s="77">
+      <c r="C7" s="76">
         <v>0</v>
       </c>
       <c r="E7" s="70" t="s">
@@ -7507,7 +7550,7 @@
       <c r="B8" s="70" t="s">
         <v>72</v>
       </c>
-      <c r="C8" s="77">
+      <c r="C8" s="76">
         <v>0</v>
       </c>
       <c r="E8" s="70" t="s">
@@ -7533,7 +7576,7 @@
       <c r="B9" s="71" t="s">
         <v>75</v>
       </c>
-      <c r="C9" s="78">
+      <c r="C9" s="77">
         <v>0</v>
       </c>
       <c r="E9" s="70" t="s">
@@ -7681,7 +7724,6 @@
       <c r="C2" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="81"/>
       <c r="E2" s="65" t="s">
         <v>19</v>
       </c>
@@ -7934,7 +7976,7 @@
         <v>150</v>
       </c>
       <c r="H17" s="23" t="s">
-        <v>80</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.3">
@@ -7971,7 +8013,9 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
       <c r="G20" s="37"/>
-      <c r="H20" s="23"/>
+      <c r="H20" s="80" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.3">
       <c r="G23" s="55"/>
@@ -11274,10 +11318,10 @@
   <sheetData>
     <row r="1" spans="1:13" ht="14.3" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:13" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="75" t="s">
+      <c r="A2" s="74" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="76">
+      <c r="B2" s="75">
         <f>SUM('Data Validation'!C5:C8)-'Data Validation'!C9</f>
         <v>0</v>
       </c>
@@ -11327,51 +11371,51 @@
         <f t="array" ref="A5:A16">Net_Salary</f>
         <v>Salary</v>
       </c>
-      <c r="B5" s="73">
+      <c r="B5" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],B$4,Tabela1[Category],$A5)</f>
         <v>0</v>
       </c>
-      <c r="C5" s="73">
+      <c r="C5" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],C$4,Tabela1[Category],$A5)</f>
         <v>0</v>
       </c>
-      <c r="D5" s="73">
+      <c r="D5" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],D$4,Tabela1[Category],$A5)</f>
         <v>0</v>
       </c>
-      <c r="E5" s="73">
+      <c r="E5" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],E$4,Tabela1[Category],$A5)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="73">
+      <c r="F5" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],F$4,Tabela1[Category],$A5)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="73">
+      <c r="G5" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],G$4,Tabela1[Category],$A5)</f>
         <v>0</v>
       </c>
-      <c r="H5" s="73">
+      <c r="H5" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],H$4,Tabela1[Category],$A5)</f>
         <v>0</v>
       </c>
-      <c r="I5" s="73">
+      <c r="I5" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],I$4,Tabela1[Category],$A5)</f>
         <v>0</v>
       </c>
-      <c r="J5" s="73">
+      <c r="J5" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],J$4,Tabela1[Category],$A5)</f>
         <v>0</v>
       </c>
-      <c r="K5" s="73">
+      <c r="K5" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],K$4,Tabela1[Category],$A5)</f>
         <v>0</v>
       </c>
-      <c r="L5" s="73">
+      <c r="L5" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],L$4,Tabela1[Category],$A5)</f>
         <v>0</v>
       </c>
-      <c r="M5" s="73">
+      <c r="M5" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],M$4,Tabela1[Category],$A5)</f>
         <v>0</v>
       </c>
@@ -11380,51 +11424,51 @@
       <c r="A6" s="30" t="str">
         <v>Seals</v>
       </c>
-      <c r="B6" s="73">
+      <c r="B6" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],B$4,Tabela1[Category],$A6)</f>
         <v>0</v>
       </c>
-      <c r="C6" s="73">
+      <c r="C6" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],C$4,Tabela1[Category],$A6)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="73">
+      <c r="D6" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],D$4,Tabela1[Category],$A6)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="73">
+      <c r="E6" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],E$4,Tabela1[Category],$A6)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="73">
+      <c r="F6" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],F$4,Tabela1[Category],$A6)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="73">
+      <c r="G6" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],G$4,Tabela1[Category],$A6)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="73">
+      <c r="H6" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],H$4,Tabela1[Category],$A6)</f>
         <v>0</v>
       </c>
-      <c r="I6" s="73">
+      <c r="I6" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],I$4,Tabela1[Category],$A6)</f>
         <v>0</v>
       </c>
-      <c r="J6" s="73">
+      <c r="J6" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],J$4,Tabela1[Category],$A6)</f>
         <v>0</v>
       </c>
-      <c r="K6" s="73">
+      <c r="K6" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],K$4,Tabela1[Category],$A6)</f>
         <v>0</v>
       </c>
-      <c r="L6" s="73">
+      <c r="L6" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],L$4,Tabela1[Category],$A6)</f>
         <v>0</v>
       </c>
-      <c r="M6" s="73">
+      <c r="M6" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],M$4,Tabela1[Category],$A6)</f>
         <v>0</v>
       </c>
@@ -11433,51 +11477,51 @@
       <c r="A7" s="30" t="str">
         <v>Rent</v>
       </c>
-      <c r="B7" s="73">
+      <c r="B7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],B$4,Tabela1[Category],$A7)</f>
         <v>0</v>
       </c>
-      <c r="C7" s="73">
+      <c r="C7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],C$4,Tabela1[Category],$A7)</f>
         <v>0</v>
       </c>
-      <c r="D7" s="73">
+      <c r="D7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],D$4,Tabela1[Category],$A7)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="73">
+      <c r="E7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],E$4,Tabela1[Category],$A7)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="73">
+      <c r="F7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],F$4,Tabela1[Category],$A7)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="73">
+      <c r="G7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],G$4,Tabela1[Category],$A7)</f>
         <v>0</v>
       </c>
-      <c r="H7" s="73">
+      <c r="H7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],H$4,Tabela1[Category],$A7)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="73">
+      <c r="I7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],I$4,Tabela1[Category],$A7)</f>
         <v>0</v>
       </c>
-      <c r="J7" s="73">
+      <c r="J7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],J$4,Tabela1[Category],$A7)</f>
         <v>0</v>
       </c>
-      <c r="K7" s="73">
+      <c r="K7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],K$4,Tabela1[Category],$A7)</f>
         <v>0</v>
       </c>
-      <c r="L7" s="73">
+      <c r="L7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],L$4,Tabela1[Category],$A7)</f>
         <v>0</v>
       </c>
-      <c r="M7" s="73">
+      <c r="M7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],M$4,Tabela1[Category],$A7)</f>
         <v>0</v>
       </c>
@@ -11486,51 +11530,51 @@
       <c r="A8" s="30" t="str">
         <v>Seals II</v>
       </c>
-      <c r="B8" s="73">
+      <c r="B8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],B$4,Tabela1[Category],$A8)</f>
         <v>0</v>
       </c>
-      <c r="C8" s="73">
+      <c r="C8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],C$4,Tabela1[Category],$A8)</f>
         <v>0</v>
       </c>
-      <c r="D8" s="73">
+      <c r="D8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],D$4,Tabela1[Category],$A8)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="73">
+      <c r="E8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],E$4,Tabela1[Category],$A8)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="73">
+      <c r="F8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],F$4,Tabela1[Category],$A8)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="73">
+      <c r="G8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],G$4,Tabela1[Category],$A8)</f>
         <v>0</v>
       </c>
-      <c r="H8" s="73">
+      <c r="H8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],H$4,Tabela1[Category],$A8)</f>
         <v>0</v>
       </c>
-      <c r="I8" s="73">
+      <c r="I8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],I$4,Tabela1[Category],$A8)</f>
         <v>0</v>
       </c>
-      <c r="J8" s="73">
+      <c r="J8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],J$4,Tabela1[Category],$A8)</f>
         <v>0</v>
       </c>
-      <c r="K8" s="73">
+      <c r="K8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],K$4,Tabela1[Category],$A8)</f>
         <v>0</v>
       </c>
-      <c r="L8" s="73">
+      <c r="L8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],L$4,Tabela1[Category],$A8)</f>
         <v>0</v>
       </c>
-      <c r="M8" s="73">
+      <c r="M8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],M$4,Tabela1[Category],$A8)</f>
         <v>0</v>
       </c>
@@ -11539,51 +11583,51 @@
       <c r="A9" s="30" t="str">
         <v>Other - Income</v>
       </c>
-      <c r="B9" s="73">
+      <c r="B9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],B$4,Tabela1[Category],$A9)</f>
         <v>0</v>
       </c>
-      <c r="C9" s="73">
+      <c r="C9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],C$4,Tabela1[Category],$A9)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="73">
+      <c r="D9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],D$4,Tabela1[Category],$A9)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="73">
+      <c r="E9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],E$4,Tabela1[Category],$A9)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="73">
+      <c r="F9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],F$4,Tabela1[Category],$A9)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="73">
+      <c r="G9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],G$4,Tabela1[Category],$A9)</f>
         <v>0</v>
       </c>
-      <c r="H9" s="73">
+      <c r="H9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],H$4,Tabela1[Category],$A9)</f>
         <v>0</v>
       </c>
-      <c r="I9" s="73">
+      <c r="I9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],I$4,Tabela1[Category],$A9)</f>
         <v>0</v>
       </c>
-      <c r="J9" s="73">
+      <c r="J9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],J$4,Tabela1[Category],$A9)</f>
         <v>0</v>
       </c>
-      <c r="K9" s="73">
+      <c r="K9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],K$4,Tabela1[Category],$A9)</f>
         <v>0</v>
       </c>
-      <c r="L9" s="73">
+      <c r="L9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],L$4,Tabela1[Category],$A9)</f>
         <v>0</v>
       </c>
-      <c r="M9" s="73">
+      <c r="M9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],M$4,Tabela1[Category],$A9)</f>
         <v>0</v>
       </c>
@@ -11592,51 +11636,51 @@
       <c r="A10" s="30" t="str">
         <v>Tax I</v>
       </c>
-      <c r="B10" s="73">
+      <c r="B10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],B$4,Tabela1[Category],$A10)</f>
         <v>0</v>
       </c>
-      <c r="C10" s="73">
+      <c r="C10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],C$4,Tabela1[Category],$A10)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="73">
+      <c r="D10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],D$4,Tabela1[Category],$A10)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="73">
+      <c r="E10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],E$4,Tabela1[Category],$A10)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="73">
+      <c r="F10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],F$4,Tabela1[Category],$A10)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="73">
+      <c r="G10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],G$4,Tabela1[Category],$A10)</f>
         <v>0</v>
       </c>
-      <c r="H10" s="73">
+      <c r="H10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],H$4,Tabela1[Category],$A10)</f>
         <v>0</v>
       </c>
-      <c r="I10" s="73">
+      <c r="I10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],I$4,Tabela1[Category],$A10)</f>
         <v>0</v>
       </c>
-      <c r="J10" s="73">
+      <c r="J10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],J$4,Tabela1[Category],$A10)</f>
         <v>0</v>
       </c>
-      <c r="K10" s="73">
+      <c r="K10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],K$4,Tabela1[Category],$A10)</f>
         <v>0</v>
       </c>
-      <c r="L10" s="73">
+      <c r="L10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],L$4,Tabela1[Category],$A10)</f>
         <v>0</v>
       </c>
-      <c r="M10" s="73">
+      <c r="M10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],M$4,Tabela1[Category],$A10)</f>
         <v>0</v>
       </c>
@@ -11645,51 +11689,51 @@
       <c r="A11" s="30" t="str">
         <v>Tax II</v>
       </c>
-      <c r="B11" s="73">
+      <c r="B11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],B$4,Tabela1[Category],$A11)</f>
         <v>0</v>
       </c>
-      <c r="C11" s="73">
+      <c r="C11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],C$4,Tabela1[Category],$A11)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="73">
+      <c r="D11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],D$4,Tabela1[Category],$A11)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="73">
+      <c r="E11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],E$4,Tabela1[Category],$A11)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="73">
+      <c r="F11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],F$4,Tabela1[Category],$A11)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="73">
+      <c r="G11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],G$4,Tabela1[Category],$A11)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="73">
+      <c r="H11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],H$4,Tabela1[Category],$A11)</f>
         <v>0</v>
       </c>
-      <c r="I11" s="73">
+      <c r="I11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],I$4,Tabela1[Category],$A11)</f>
         <v>0</v>
       </c>
-      <c r="J11" s="73">
+      <c r="J11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],J$4,Tabela1[Category],$A11)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="73">
+      <c r="K11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],K$4,Tabela1[Category],$A11)</f>
         <v>0</v>
       </c>
-      <c r="L11" s="73">
+      <c r="L11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],L$4,Tabela1[Category],$A11)</f>
         <v>0</v>
       </c>
-      <c r="M11" s="73">
+      <c r="M11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],M$4,Tabela1[Category],$A11)</f>
         <v>0</v>
       </c>
@@ -11698,51 +11742,51 @@
       <c r="A12" s="30" t="str">
         <v>Bank Fee I</v>
       </c>
-      <c r="B12" s="73">
+      <c r="B12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],B$4,Tabela1[Category],$A12)</f>
         <v>0</v>
       </c>
-      <c r="C12" s="73">
+      <c r="C12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],C$4,Tabela1[Category],$A12)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="73">
+      <c r="D12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],D$4,Tabela1[Category],$A12)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="73">
+      <c r="E12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],E$4,Tabela1[Category],$A12)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="73">
+      <c r="F12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],F$4,Tabela1[Category],$A12)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="73">
+      <c r="G12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],G$4,Tabela1[Category],$A12)</f>
         <v>0</v>
       </c>
-      <c r="H12" s="73">
+      <c r="H12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],H$4,Tabela1[Category],$A12)</f>
         <v>0</v>
       </c>
-      <c r="I12" s="73">
+      <c r="I12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],I$4,Tabela1[Category],$A12)</f>
         <v>0</v>
       </c>
-      <c r="J12" s="73">
+      <c r="J12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],J$4,Tabela1[Category],$A12)</f>
         <v>0</v>
       </c>
-      <c r="K12" s="73">
+      <c r="K12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],K$4,Tabela1[Category],$A12)</f>
         <v>0</v>
       </c>
-      <c r="L12" s="73">
+      <c r="L12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],L$4,Tabela1[Category],$A12)</f>
         <v>0</v>
       </c>
-      <c r="M12" s="73">
+      <c r="M12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],M$4,Tabela1[Category],$A12)</f>
         <v>0</v>
       </c>
@@ -11751,51 +11795,51 @@
       <c r="A13" s="30" t="str">
         <v>Bank Fee II</v>
       </c>
-      <c r="B13" s="73">
+      <c r="B13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],B$4,Tabela1[Category],$A13)</f>
         <v>0</v>
       </c>
-      <c r="C13" s="73">
+      <c r="C13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],C$4,Tabela1[Category],$A13)</f>
         <v>0</v>
       </c>
-      <c r="D13" s="73">
+      <c r="D13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],D$4,Tabela1[Category],$A13)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="73">
+      <c r="E13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],E$4,Tabela1[Category],$A13)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="73">
+      <c r="F13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],F$4,Tabela1[Category],$A13)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="73">
+      <c r="G13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],G$4,Tabela1[Category],$A13)</f>
         <v>0</v>
       </c>
-      <c r="H13" s="73">
+      <c r="H13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],H$4,Tabela1[Category],$A13)</f>
         <v>0</v>
       </c>
-      <c r="I13" s="73">
+      <c r="I13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],I$4,Tabela1[Category],$A13)</f>
         <v>0</v>
       </c>
-      <c r="J13" s="73">
+      <c r="J13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],J$4,Tabela1[Category],$A13)</f>
         <v>0</v>
       </c>
-      <c r="K13" s="73">
+      <c r="K13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],K$4,Tabela1[Category],$A13)</f>
         <v>0</v>
       </c>
-      <c r="L13" s="73">
+      <c r="L13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],L$4,Tabela1[Category],$A13)</f>
         <v>0</v>
       </c>
-      <c r="M13" s="73">
+      <c r="M13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],M$4,Tabela1[Category],$A13)</f>
         <v>0</v>
       </c>
@@ -11804,51 +11848,51 @@
       <c r="A14" s="30" t="str">
         <v>Other - Discount</v>
       </c>
-      <c r="B14" s="73">
+      <c r="B14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],B$4,Tabela1[Category],$A14)</f>
         <v>0</v>
       </c>
-      <c r="C14" s="73">
+      <c r="C14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],C$4,Tabela1[Category],$A14)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="73">
+      <c r="D14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],D$4,Tabela1[Category],$A14)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="73">
+      <c r="E14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],E$4,Tabela1[Category],$A14)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="73">
+      <c r="F14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],F$4,Tabela1[Category],$A14)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="73">
+      <c r="G14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],G$4,Tabela1[Category],$A14)</f>
         <v>0</v>
       </c>
-      <c r="H14" s="73">
+      <c r="H14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],H$4,Tabela1[Category],$A14)</f>
         <v>0</v>
       </c>
-      <c r="I14" s="73">
+      <c r="I14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],I$4,Tabela1[Category],$A14)</f>
         <v>0</v>
       </c>
-      <c r="J14" s="73">
+      <c r="J14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],J$4,Tabela1[Category],$A14)</f>
         <v>0</v>
       </c>
-      <c r="K14" s="73">
+      <c r="K14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],K$4,Tabela1[Category],$A14)</f>
         <v>0</v>
       </c>
-      <c r="L14" s="73">
+      <c r="L14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],L$4,Tabela1[Category],$A14)</f>
         <v>0</v>
       </c>
-      <c r="M14" s="73">
+      <c r="M14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],M$4,Tabela1[Category],$A14)</f>
         <v>0</v>
       </c>
@@ -11857,51 +11901,51 @@
       <c r="A15" s="30" t="str">
         <v>Stock Market</v>
       </c>
-      <c r="B15" s="73">
+      <c r="B15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],B$4,Tabela1[Category],$A15)</f>
         <v>0</v>
       </c>
-      <c r="C15" s="73">
+      <c r="C15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],C$4,Tabela1[Category],$A15)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="73">
+      <c r="D15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],D$4,Tabela1[Category],$A15)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="73">
+      <c r="E15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],E$4,Tabela1[Category],$A15)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="73">
+      <c r="F15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],F$4,Tabela1[Category],$A15)</f>
         <v>0</v>
       </c>
-      <c r="G15" s="73">
+      <c r="G15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],G$4,Tabela1[Category],$A15)</f>
         <v>0</v>
       </c>
-      <c r="H15" s="73">
+      <c r="H15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],H$4,Tabela1[Category],$A15)</f>
         <v>0</v>
       </c>
-      <c r="I15" s="73">
+      <c r="I15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],I$4,Tabela1[Category],$A15)</f>
         <v>0</v>
       </c>
-      <c r="J15" s="73">
+      <c r="J15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],J$4,Tabela1[Category],$A15)</f>
         <v>0</v>
       </c>
-      <c r="K15" s="73">
+      <c r="K15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],K$4,Tabela1[Category],$A15)</f>
         <v>0</v>
       </c>
-      <c r="L15" s="73">
+      <c r="L15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],L$4,Tabela1[Category],$A15)</f>
         <v>0</v>
       </c>
-      <c r="M15" s="73">
+      <c r="M15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],M$4,Tabela1[Category],$A15)</f>
         <v>0</v>
       </c>
@@ -11910,51 +11954,51 @@
       <c r="A16" s="30" t="str">
         <v>Real Estate</v>
       </c>
-      <c r="B16" s="73">
+      <c r="B16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],B$4,Tabela1[Category],$A16)</f>
         <v>0</v>
       </c>
-      <c r="C16" s="73">
+      <c r="C16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],C$4,Tabela1[Category],$A16)</f>
         <v>0</v>
       </c>
-      <c r="D16" s="73">
+      <c r="D16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],D$4,Tabela1[Category],$A16)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="73">
+      <c r="E16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],E$4,Tabela1[Category],$A16)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="73">
+      <c r="F16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],F$4,Tabela1[Category],$A16)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="73">
+      <c r="G16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],G$4,Tabela1[Category],$A16)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="73">
+      <c r="H16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],H$4,Tabela1[Category],$A16)</f>
         <v>0</v>
       </c>
-      <c r="I16" s="73">
+      <c r="I16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],I$4,Tabela1[Category],$A16)</f>
         <v>0</v>
       </c>
-      <c r="J16" s="73">
+      <c r="J16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],J$4,Tabela1[Category],$A16)</f>
         <v>0</v>
       </c>
-      <c r="K16" s="73">
+      <c r="K16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],K$4,Tabela1[Category],$A16)</f>
         <v>0</v>
       </c>
-      <c r="L16" s="73">
+      <c r="L16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],L$4,Tabela1[Category],$A16)</f>
         <v>0</v>
       </c>
-      <c r="M16" s="73">
+      <c r="M16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],M$4,Tabela1[Category],$A16)</f>
         <v>0</v>
       </c>
@@ -12133,107 +12177,107 @@
       </c>
     </row>
     <row r="3" spans="1:13" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="72" t="s">
+      <c r="A3" s="89" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="73">
+      <c r="B3" s="72">
         <f>'Net Salary'!B18</f>
         <v>0</v>
       </c>
-      <c r="C3" s="73">
+      <c r="C3" s="72">
         <f>'Net Salary'!C18</f>
         <v>0</v>
       </c>
-      <c r="D3" s="73">
+      <c r="D3" s="72">
         <f>'Net Salary'!D18</f>
         <v>0</v>
       </c>
-      <c r="E3" s="73">
+      <c r="E3" s="72">
         <f>'Net Salary'!E18</f>
         <v>0</v>
       </c>
-      <c r="F3" s="73">
+      <c r="F3" s="72">
         <f>'Net Salary'!F18</f>
         <v>0</v>
       </c>
-      <c r="G3" s="73">
+      <c r="G3" s="72">
         <f>'Net Salary'!G18</f>
         <v>0</v>
       </c>
-      <c r="H3" s="73">
+      <c r="H3" s="72">
         <f>'Net Salary'!H18</f>
         <v>0</v>
       </c>
-      <c r="I3" s="73">
+      <c r="I3" s="72">
         <f>'Net Salary'!I18</f>
         <v>0</v>
       </c>
-      <c r="J3" s="73">
+      <c r="J3" s="72">
         <f>'Net Salary'!J18</f>
         <v>0</v>
       </c>
-      <c r="K3" s="73">
+      <c r="K3" s="72">
         <f>'Net Salary'!K18</f>
         <v>0</v>
       </c>
-      <c r="L3" s="73">
+      <c r="L3" s="72">
         <f>'Net Salary'!L18</f>
         <v>0</v>
       </c>
-      <c r="M3" s="73">
+      <c r="M3" s="72">
         <f>'Net Salary'!M18</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="72" t="s">
+      <c r="A4" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="74">
+      <c r="B4" s="73">
         <f>B3-(SUM(B7:B18))</f>
         <v>0</v>
       </c>
-      <c r="C4" s="74">
+      <c r="C4" s="73">
         <f t="shared" ref="C4:L4" si="0">C3-(SUM(C7:C18))+B4</f>
         <v>0</v>
       </c>
-      <c r="D4" s="74">
+      <c r="D4" s="73">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E4" s="74">
+      <c r="E4" s="73">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F4" s="74">
+      <c r="F4" s="73">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G4" s="74">
+      <c r="G4" s="73">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H4" s="74">
+      <c r="H4" s="73">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I4" s="74">
+      <c r="I4" s="73">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J4" s="74">
+      <c r="J4" s="73">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K4" s="74">
+      <c r="K4" s="73">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L4" s="74">
+      <c r="L4" s="73">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M4" s="74">
+      <c r="M4" s="73">
         <f>M3-SUM(M7:M18)+L4</f>
         <v>0</v>
       </c>
@@ -12299,51 +12343,51 @@
         <f t="array" ref="A7:A18">Expenses</f>
         <v>Bills</v>
       </c>
-      <c r="B7" s="73">
+      <c r="B7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!B$2,Tabela1[Category],Expenses!$A7)</f>
         <v>0</v>
       </c>
-      <c r="C7" s="73">
+      <c r="C7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!C$2,Tabela1[Category],Expenses!$A7)</f>
         <v>0</v>
       </c>
-      <c r="D7" s="73">
+      <c r="D7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!D$2,Tabela1[Category],Expenses!$A7)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="73">
+      <c r="E7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!E$2,Tabela1[Category],Expenses!$A7)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="73">
+      <c r="F7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!F$2,Tabela1[Category],Expenses!$A7)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="73">
+      <c r="G7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!G$2,Tabela1[Category],Expenses!$A7)</f>
         <v>0</v>
       </c>
-      <c r="H7" s="73">
+      <c r="H7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!H$2,Tabela1[Category],Expenses!$A7)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="73">
+      <c r="I7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!I$2,Tabela1[Category],Expenses!$A7)</f>
         <v>0</v>
       </c>
-      <c r="J7" s="73">
+      <c r="J7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!J$2,Tabela1[Category],Expenses!$A7)</f>
         <v>0</v>
       </c>
-      <c r="K7" s="73">
+      <c r="K7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!K$2,Tabela1[Category],Expenses!$A7)</f>
         <v>0</v>
       </c>
-      <c r="L7" s="73">
+      <c r="L7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!L$2,Tabela1[Category],Expenses!$A7)</f>
         <v>0</v>
       </c>
-      <c r="M7" s="73">
+      <c r="M7" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!M$2,Tabela1[Category],Expenses!$A7)</f>
         <v>0</v>
       </c>
@@ -12352,51 +12396,51 @@
       <c r="A8" s="15" t="str">
         <v xml:space="preserve">Car </v>
       </c>
-      <c r="B8" s="73">
+      <c r="B8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!B$2,Tabela1[Category],Expenses!$A8)</f>
         <v>0</v>
       </c>
-      <c r="C8" s="73">
+      <c r="C8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!C$2,Tabela1[Category],Expenses!$A8)</f>
         <v>0</v>
       </c>
-      <c r="D8" s="73">
+      <c r="D8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!D$2,Tabela1[Category],Expenses!$A8)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="73">
+      <c r="E8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!E$2,Tabela1[Category],Expenses!$A8)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="73">
+      <c r="F8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!F$2,Tabela1[Category],Expenses!$A8)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="73">
+      <c r="G8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!G$2,Tabela1[Category],Expenses!$A8)</f>
         <v>0</v>
       </c>
-      <c r="H8" s="73">
+      <c r="H8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!H$2,Tabela1[Category],Expenses!$A8)</f>
         <v>0</v>
       </c>
-      <c r="I8" s="73">
+      <c r="I8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!I$2,Tabela1[Category],Expenses!$A8)</f>
         <v>0</v>
       </c>
-      <c r="J8" s="73">
+      <c r="J8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!J$2,Tabela1[Category],Expenses!$A8)</f>
         <v>0</v>
       </c>
-      <c r="K8" s="73">
+      <c r="K8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!K$2,Tabela1[Category],Expenses!$A8)</f>
         <v>0</v>
       </c>
-      <c r="L8" s="73">
+      <c r="L8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!L$2,Tabela1[Category],Expenses!$A8)</f>
         <v>0</v>
       </c>
-      <c r="M8" s="73">
+      <c r="M8" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!M$2,Tabela1[Category],Expenses!$A8)</f>
         <v>0</v>
       </c>
@@ -12405,51 +12449,51 @@
       <c r="A9" s="15" t="str">
         <v>Clothing</v>
       </c>
-      <c r="B9" s="73">
+      <c r="B9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!B$2,Tabela1[Category],Expenses!$A9)</f>
         <v>0</v>
       </c>
-      <c r="C9" s="73">
+      <c r="C9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!C$2,Tabela1[Category],Expenses!$A9)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="73">
+      <c r="D9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!D$2,Tabela1[Category],Expenses!$A9)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="73">
+      <c r="E9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!E$2,Tabela1[Category],Expenses!$A9)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="73">
+      <c r="F9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!F$2,Tabela1[Category],Expenses!$A9)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="73">
+      <c r="G9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!G$2,Tabela1[Category],Expenses!$A9)</f>
         <v>0</v>
       </c>
-      <c r="H9" s="73">
+      <c r="H9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!H$2,Tabela1[Category],Expenses!$A9)</f>
         <v>0</v>
       </c>
-      <c r="I9" s="73">
+      <c r="I9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!I$2,Tabela1[Category],Expenses!$A9)</f>
         <v>0</v>
       </c>
-      <c r="J9" s="73">
+      <c r="J9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!J$2,Tabela1[Category],Expenses!$A9)</f>
         <v>0</v>
       </c>
-      <c r="K9" s="73">
+      <c r="K9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!K$2,Tabela1[Category],Expenses!$A9)</f>
         <v>0</v>
       </c>
-      <c r="L9" s="73">
+      <c r="L9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!L$2,Tabela1[Category],Expenses!$A9)</f>
         <v>0</v>
       </c>
-      <c r="M9" s="73">
+      <c r="M9" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!M$2,Tabela1[Category],Expenses!$A9)</f>
         <v>0</v>
       </c>
@@ -12458,51 +12502,51 @@
       <c r="A10" s="15" t="str">
         <v>Eletron n' games</v>
       </c>
-      <c r="B10" s="73">
+      <c r="B10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!B$2,Tabela1[Category],Expenses!$A10)</f>
         <v>0</v>
       </c>
-      <c r="C10" s="73">
+      <c r="C10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!C$2,Tabela1[Category],Expenses!$A10)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="73">
+      <c r="D10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!D$2,Tabela1[Category],Expenses!$A10)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="73">
+      <c r="E10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!E$2,Tabela1[Category],Expenses!$A10)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="73">
+      <c r="F10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!F$2,Tabela1[Category],Expenses!$A10)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="73">
+      <c r="G10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!G$2,Tabela1[Category],Expenses!$A10)</f>
         <v>0</v>
       </c>
-      <c r="H10" s="73">
+      <c r="H10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!H$2,Tabela1[Category],Expenses!$A10)</f>
         <v>0</v>
       </c>
-      <c r="I10" s="73">
+      <c r="I10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!I$2,Tabela1[Category],Expenses!$A10)</f>
         <v>0</v>
       </c>
-      <c r="J10" s="73">
+      <c r="J10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!J$2,Tabela1[Category],Expenses!$A10)</f>
         <v>0</v>
       </c>
-      <c r="K10" s="73">
+      <c r="K10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!K$2,Tabela1[Category],Expenses!$A10)</f>
         <v>0</v>
       </c>
-      <c r="L10" s="73">
+      <c r="L10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!L$2,Tabela1[Category],Expenses!$A10)</f>
         <v>0</v>
       </c>
-      <c r="M10" s="73">
+      <c r="M10" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!M$2,Tabela1[Category],Expenses!$A10)</f>
         <v>0</v>
       </c>
@@ -12511,51 +12555,51 @@
       <c r="A11" s="15" t="str">
         <v>Food</v>
       </c>
-      <c r="B11" s="73">
+      <c r="B11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!B$2,Tabela1[Category],Expenses!$A11)</f>
         <v>0</v>
       </c>
-      <c r="C11" s="73">
+      <c r="C11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!C$2,Tabela1[Category],Expenses!$A11)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="73">
+      <c r="D11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!D$2,Tabela1[Category],Expenses!$A11)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="73">
+      <c r="E11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!E$2,Tabela1[Category],Expenses!$A11)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="73">
+      <c r="F11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!F$2,Tabela1[Category],Expenses!$A11)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="73">
+      <c r="G11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!G$2,Tabela1[Category],Expenses!$A11)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="73">
+      <c r="H11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!H$2,Tabela1[Category],Expenses!$A11)</f>
         <v>0</v>
       </c>
-      <c r="I11" s="73">
+      <c r="I11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!I$2,Tabela1[Category],Expenses!$A11)</f>
         <v>0</v>
       </c>
-      <c r="J11" s="73">
+      <c r="J11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!J$2,Tabela1[Category],Expenses!$A11)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="73">
+      <c r="K11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!K$2,Tabela1[Category],Expenses!$A11)</f>
         <v>0</v>
       </c>
-      <c r="L11" s="73">
+      <c r="L11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!L$2,Tabela1[Category],Expenses!$A11)</f>
         <v>0</v>
       </c>
-      <c r="M11" s="73">
+      <c r="M11" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!M$2,Tabela1[Category],Expenses!$A11)</f>
         <v>0</v>
       </c>
@@ -12564,51 +12608,51 @@
       <c r="A12" s="15" t="str">
         <v>Gasolina</v>
       </c>
-      <c r="B12" s="73">
+      <c r="B12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!B$2,Tabela1[Category],Expenses!$A12)</f>
         <v>0</v>
       </c>
-      <c r="C12" s="73">
+      <c r="C12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!C$2,Tabela1[Category],Expenses!$A12)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="73">
+      <c r="D12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!D$2,Tabela1[Category],Expenses!$A12)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="73">
+      <c r="E12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!E$2,Tabela1[Category],Expenses!$A12)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="73">
+      <c r="F12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!F$2,Tabela1[Category],Expenses!$A12)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="73">
+      <c r="G12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!G$2,Tabela1[Category],Expenses!$A12)</f>
         <v>0</v>
       </c>
-      <c r="H12" s="73">
+      <c r="H12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!H$2,Tabela1[Category],Expenses!$A12)</f>
         <v>0</v>
       </c>
-      <c r="I12" s="73">
+      <c r="I12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!I$2,Tabela1[Category],Expenses!$A12)</f>
         <v>0</v>
       </c>
-      <c r="J12" s="73">
+      <c r="J12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!J$2,Tabela1[Category],Expenses!$A12)</f>
         <v>0</v>
       </c>
-      <c r="K12" s="73">
+      <c r="K12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!K$2,Tabela1[Category],Expenses!$A12)</f>
         <v>0</v>
       </c>
-      <c r="L12" s="73">
+      <c r="L12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!L$2,Tabela1[Category],Expenses!$A12)</f>
         <v>0</v>
       </c>
-      <c r="M12" s="73">
+      <c r="M12" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!M$2,Tabela1[Category],Expenses!$A12)</f>
         <v>0</v>
       </c>
@@ -12617,51 +12661,51 @@
       <c r="A13" s="15" t="str">
         <v>Hang out</v>
       </c>
-      <c r="B13" s="73">
+      <c r="B13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!B$2,Tabela1[Category],Expenses!$A13)</f>
         <v>0</v>
       </c>
-      <c r="C13" s="73">
+      <c r="C13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!C$2,Tabela1[Category],Expenses!$A13)</f>
         <v>0</v>
       </c>
-      <c r="D13" s="73">
+      <c r="D13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!D$2,Tabela1[Category],Expenses!$A13)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="73">
+      <c r="E13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!E$2,Tabela1[Category],Expenses!$A13)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="73">
+      <c r="F13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!F$2,Tabela1[Category],Expenses!$A13)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="73">
+      <c r="G13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!G$2,Tabela1[Category],Expenses!$A13)</f>
         <v>0</v>
       </c>
-      <c r="H13" s="73">
+      <c r="H13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!H$2,Tabela1[Category],Expenses!$A13)</f>
         <v>0</v>
       </c>
-      <c r="I13" s="73">
+      <c r="I13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!I$2,Tabela1[Category],Expenses!$A13)</f>
         <v>0</v>
       </c>
-      <c r="J13" s="73">
+      <c r="J13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!J$2,Tabela1[Category],Expenses!$A13)</f>
         <v>0</v>
       </c>
-      <c r="K13" s="73">
+      <c r="K13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!K$2,Tabela1[Category],Expenses!$A13)</f>
         <v>0</v>
       </c>
-      <c r="L13" s="73">
+      <c r="L13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!L$2,Tabela1[Category],Expenses!$A13)</f>
         <v>0</v>
       </c>
-      <c r="M13" s="73">
+      <c r="M13" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!M$2,Tabela1[Category],Expenses!$A13)</f>
         <v>0</v>
       </c>
@@ -12670,51 +12714,51 @@
       <c r="A14" s="51" t="str">
         <v>Healthcare</v>
       </c>
-      <c r="B14" s="73">
+      <c r="B14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!B$2,Tabela1[Category],Expenses!$A14)</f>
         <v>0</v>
       </c>
-      <c r="C14" s="73">
+      <c r="C14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!C$2,Tabela1[Category],Expenses!$A14)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="73">
+      <c r="D14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!D$2,Tabela1[Category],Expenses!$A14)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="73">
+      <c r="E14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!E$2,Tabela1[Category],Expenses!$A14)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="73">
+      <c r="F14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!F$2,Tabela1[Category],Expenses!$A14)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="73">
+      <c r="G14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!G$2,Tabela1[Category],Expenses!$A14)</f>
         <v>0</v>
       </c>
-      <c r="H14" s="73">
+      <c r="H14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!H$2,Tabela1[Category],Expenses!$A14)</f>
         <v>0</v>
       </c>
-      <c r="I14" s="73">
+      <c r="I14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!I$2,Tabela1[Category],Expenses!$A14)</f>
         <v>0</v>
       </c>
-      <c r="J14" s="73">
+      <c r="J14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!J$2,Tabela1[Category],Expenses!$A14)</f>
         <v>0</v>
       </c>
-      <c r="K14" s="73">
+      <c r="K14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!K$2,Tabela1[Category],Expenses!$A14)</f>
         <v>0</v>
       </c>
-      <c r="L14" s="73">
+      <c r="L14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!L$2,Tabela1[Category],Expenses!$A14)</f>
         <v>0</v>
       </c>
-      <c r="M14" s="73">
+      <c r="M14" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!M$2,Tabela1[Category],Expenses!$A14)</f>
         <v>0</v>
       </c>
@@ -12723,51 +12767,51 @@
       <c r="A15" s="15" t="str">
         <v>Insurance</v>
       </c>
-      <c r="B15" s="73">
+      <c r="B15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!B$2,Tabela1[Category],Expenses!$A15)</f>
         <v>0</v>
       </c>
-      <c r="C15" s="73">
+      <c r="C15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!C$2,Tabela1[Category],Expenses!$A15)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="73">
+      <c r="D15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!D$2,Tabela1[Category],Expenses!$A15)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="73">
+      <c r="E15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!E$2,Tabela1[Category],Expenses!$A15)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="73">
+      <c r="F15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!F$2,Tabela1[Category],Expenses!$A15)</f>
         <v>0</v>
       </c>
-      <c r="G15" s="73">
+      <c r="G15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!G$2,Tabela1[Category],Expenses!$A15)</f>
         <v>0</v>
       </c>
-      <c r="H15" s="73">
+      <c r="H15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!H$2,Tabela1[Category],Expenses!$A15)</f>
         <v>0</v>
       </c>
-      <c r="I15" s="73">
+      <c r="I15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!I$2,Tabela1[Category],Expenses!$A15)</f>
         <v>0</v>
       </c>
-      <c r="J15" s="73">
+      <c r="J15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!J$2,Tabela1[Category],Expenses!$A15)</f>
         <v>0</v>
       </c>
-      <c r="K15" s="73">
+      <c r="K15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!K$2,Tabela1[Category],Expenses!$A15)</f>
         <v>0</v>
       </c>
-      <c r="L15" s="73">
+      <c r="L15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!L$2,Tabela1[Category],Expenses!$A15)</f>
         <v>0</v>
       </c>
-      <c r="M15" s="73">
+      <c r="M15" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!M$2,Tabela1[Category],Expenses!$A15)</f>
         <v>0</v>
       </c>
@@ -12776,51 +12820,51 @@
       <c r="A16" s="15" t="str">
         <v>Personal Care</v>
       </c>
-      <c r="B16" s="73">
+      <c r="B16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!B$2,Tabela1[Category],Expenses!$A16)</f>
         <v>0</v>
       </c>
-      <c r="C16" s="73">
+      <c r="C16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!C$2,Tabela1[Category],Expenses!$A16)</f>
         <v>0</v>
       </c>
-      <c r="D16" s="73">
+      <c r="D16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!D$2,Tabela1[Category],Expenses!$A16)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="73">
+      <c r="E16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!E$2,Tabela1[Category],Expenses!$A16)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="73">
+      <c r="F16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!F$2,Tabela1[Category],Expenses!$A16)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="73">
+      <c r="G16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!G$2,Tabela1[Category],Expenses!$A16)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="73">
+      <c r="H16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!H$2,Tabela1[Category],Expenses!$A16)</f>
         <v>0</v>
       </c>
-      <c r="I16" s="73">
+      <c r="I16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!I$2,Tabela1[Category],Expenses!$A16)</f>
         <v>0</v>
       </c>
-      <c r="J16" s="73">
+      <c r="J16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!J$2,Tabela1[Category],Expenses!$A16)</f>
         <v>0</v>
       </c>
-      <c r="K16" s="73">
+      <c r="K16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!K$2,Tabela1[Category],Expenses!$A16)</f>
         <v>0</v>
       </c>
-      <c r="L16" s="73">
+      <c r="L16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!L$2,Tabela1[Category],Expenses!$A16)</f>
         <v>0</v>
       </c>
-      <c r="M16" s="73">
+      <c r="M16" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!M$2,Tabela1[Category],Expenses!$A16)</f>
         <v>0</v>
       </c>
@@ -12829,51 +12873,51 @@
       <c r="A17" s="15" t="str">
         <v>Travel</v>
       </c>
-      <c r="B17" s="73">
+      <c r="B17" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!B$2,Tabela1[Category],Expenses!$A17)</f>
         <v>0</v>
       </c>
-      <c r="C17" s="73">
+      <c r="C17" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!C$2,Tabela1[Category],Expenses!$A17)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="73">
+      <c r="D17" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!D$2,Tabela1[Category],Expenses!$A17)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="73">
+      <c r="E17" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!E$2,Tabela1[Category],Expenses!$A17)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="73">
+      <c r="F17" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!F$2,Tabela1[Category],Expenses!$A17)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="73">
+      <c r="G17" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!G$2,Tabela1[Category],Expenses!$A17)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="73">
+      <c r="H17" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!H$2,Tabela1[Category],Expenses!$A17)</f>
         <v>0</v>
       </c>
-      <c r="I17" s="73">
+      <c r="I17" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!I$2,Tabela1[Category],Expenses!$A17)</f>
         <v>0</v>
       </c>
-      <c r="J17" s="73">
+      <c r="J17" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!J$2,Tabela1[Category],Expenses!$A17)</f>
         <v>0</v>
       </c>
-      <c r="K17" s="73">
+      <c r="K17" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!K$2,Tabela1[Category],Expenses!$A17)</f>
         <v>0</v>
       </c>
-      <c r="L17" s="73">
+      <c r="L17" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!L$2,Tabela1[Category],Expenses!$A17)</f>
         <v>0</v>
       </c>
-      <c r="M17" s="73">
+      <c r="M17" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!M$2,Tabela1[Category],Expenses!$A17)</f>
         <v>0</v>
       </c>
@@ -12882,51 +12926,51 @@
       <c r="A18" s="15" t="str">
         <v>General expen.</v>
       </c>
-      <c r="B18" s="73">
+      <c r="B18" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!B$2,Tabela1[Category],Expenses!$A18)</f>
         <v>0</v>
       </c>
-      <c r="C18" s="73">
+      <c r="C18" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!C$2,Tabela1[Category],Expenses!$A18)</f>
         <v>0</v>
       </c>
-      <c r="D18" s="73">
+      <c r="D18" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!D$2,Tabela1[Category],Expenses!$A18)</f>
         <v>0</v>
       </c>
-      <c r="E18" s="73">
+      <c r="E18" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!E$2,Tabela1[Category],Expenses!$A18)</f>
         <v>0</v>
       </c>
-      <c r="F18" s="73">
+      <c r="F18" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!F$2,Tabela1[Category],Expenses!$A18)</f>
         <v>0</v>
       </c>
-      <c r="G18" s="73">
+      <c r="G18" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!G$2,Tabela1[Category],Expenses!$A18)</f>
         <v>0</v>
       </c>
-      <c r="H18" s="73">
+      <c r="H18" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!H$2,Tabela1[Category],Expenses!$A18)</f>
         <v>0</v>
       </c>
-      <c r="I18" s="73">
+      <c r="I18" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!I$2,Tabela1[Category],Expenses!$A18)</f>
         <v>0</v>
       </c>
-      <c r="J18" s="73">
+      <c r="J18" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!J$2,Tabela1[Category],Expenses!$A18)</f>
         <v>0</v>
       </c>
-      <c r="K18" s="73">
+      <c r="K18" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!K$2,Tabela1[Category],Expenses!$A18)</f>
         <v>0</v>
       </c>
-      <c r="L18" s="73">
+      <c r="L18" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!L$2,Tabela1[Category],Expenses!$A18)</f>
         <v>0</v>
       </c>
-      <c r="M18" s="73">
+      <c r="M18" s="72">
         <f>SUMIFS(Tabela1[Amount],Tabela1[Month],Expenses!M$2,Tabela1[Category],Expenses!$A18)</f>
         <v>0</v>
       </c>
@@ -13026,6 +13070,2617 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FE8D062-9855-4AFA-B18C-684CE2F5E950}">
+  <dimension ref="B2:L202"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="81"/>
+    <col min="2" max="2" width="14.28515625" style="81" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" style="81" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="81"/>
+    <col min="5" max="6" width="10.7109375" style="81" customWidth="1"/>
+    <col min="7" max="8" width="14.28515625" style="81" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" style="81" customWidth="1"/>
+    <col min="10" max="11" width="14.28515625" style="81" customWidth="1"/>
+    <col min="12" max="12" width="28.5703125" style="81" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="81"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12" ht="14.3" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="28" t="s">
+        <v>86</v>
+      </c>
+      <c r="F2" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="K2" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="28" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B3" s="67" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="36">
+        <f>MAX($K$3:$K$185)</f>
+        <v>150</v>
+      </c>
+      <c r="E3" s="82">
+        <v>0</v>
+      </c>
+      <c r="F3" s="83" cm="1">
+        <f t="array" ref="F3:L3">_xlfn._xlws.SORT(_xlfn._xlws.FILTER(Tabela1[],Tabela1[Description]=C2),1,1,FALSE)</f>
+        <v>45292</v>
+      </c>
+      <c r="G3" s="82" t="str">
+        <v>Janeiro</v>
+      </c>
+      <c r="H3" s="82" t="str">
+        <v>Income</v>
+      </c>
+      <c r="I3" s="82" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="J3" s="82" t="str">
+        <v>Bank 1</v>
+      </c>
+      <c r="K3" s="90">
+        <v>150</v>
+      </c>
+      <c r="L3" s="82" t="str">
+        <v>Salary</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B4" s="67" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="36">
+        <f>MIN($K$3:$K$185)</f>
+        <v>150</v>
+      </c>
+      <c r="E4" s="82" t="str">
+        <f>IF(ISBLANK(F4),"",F4-F3)</f>
+        <v/>
+      </c>
+      <c r="F4" s="83"/>
+      <c r="G4" s="82"/>
+      <c r="H4" s="82"/>
+      <c r="I4" s="82"/>
+      <c r="J4" s="82"/>
+      <c r="K4" s="90"/>
+      <c r="L4" s="82"/>
+    </row>
+    <row r="5" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B5" s="67" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="36">
+        <f>AVERAGE($K$3:$K$185)</f>
+        <v>150</v>
+      </c>
+      <c r="E5" s="82" t="str">
+        <f t="shared" ref="E5:E68" si="0">IF(ISBLANK(F5),"",F5-F4)</f>
+        <v/>
+      </c>
+      <c r="F5" s="83"/>
+      <c r="G5" s="82"/>
+      <c r="H5" s="82"/>
+      <c r="I5" s="82"/>
+      <c r="J5" s="82"/>
+      <c r="K5" s="90"/>
+      <c r="L5" s="82"/>
+    </row>
+    <row r="6" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B6" s="67" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="36">
+        <f>SUM($K$3:$K$185)</f>
+        <v>150</v>
+      </c>
+      <c r="E6" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F6" s="83"/>
+      <c r="G6" s="82"/>
+      <c r="H6" s="82"/>
+      <c r="I6" s="82"/>
+      <c r="J6" s="82"/>
+      <c r="K6" s="90"/>
+      <c r="L6" s="82"/>
+    </row>
+    <row r="7" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B7" s="67" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="82">
+        <f>SUBTOTAL(2,F3:F185)</f>
+        <v>1</v>
+      </c>
+      <c r="E7" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F7" s="83"/>
+      <c r="G7" s="82"/>
+      <c r="H7" s="82"/>
+      <c r="I7" s="82"/>
+      <c r="J7" s="82"/>
+      <c r="K7" s="90"/>
+      <c r="L7" s="82"/>
+    </row>
+    <row r="8" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B8" s="67" t="s">
+        <v>82</v>
+      </c>
+      <c r="C8" s="84" t="str">
+        <f>IFERROR(AVERAGE($E$4:$E$185)+MAX($F$3:$F$185),"No data.")</f>
+        <v>No data.</v>
+      </c>
+      <c r="E8" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F8" s="83"/>
+      <c r="G8" s="82"/>
+      <c r="H8" s="82"/>
+      <c r="I8" s="82"/>
+      <c r="J8" s="82"/>
+      <c r="K8" s="90"/>
+      <c r="L8" s="82"/>
+    </row>
+    <row r="9" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E9" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F9" s="83"/>
+      <c r="G9" s="82"/>
+      <c r="H9" s="82"/>
+      <c r="I9" s="82"/>
+      <c r="J9" s="82"/>
+      <c r="K9" s="90"/>
+      <c r="L9" s="82"/>
+    </row>
+    <row r="10" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B10" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F10" s="83"/>
+      <c r="G10" s="82"/>
+      <c r="H10" s="82"/>
+      <c r="I10" s="82"/>
+      <c r="J10" s="82"/>
+      <c r="K10" s="90"/>
+      <c r="L10" s="82"/>
+    </row>
+    <row r="11" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B11" s="67" t="str" cm="1">
+        <f t="array" ref="B11:B22">Months</f>
+        <v>January</v>
+      </c>
+      <c r="C11" s="88">
+        <f t="shared" ref="C11:C22" si="1">SUMIFS($K$3:$K$185,$G$3:$G$185,B11,$L$3:$L$185,$C$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F11" s="83"/>
+      <c r="G11" s="82"/>
+      <c r="H11" s="82"/>
+      <c r="I11" s="82"/>
+      <c r="J11" s="82"/>
+      <c r="K11" s="90"/>
+      <c r="L11" s="82"/>
+    </row>
+    <row r="12" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B12" s="67" t="str">
+        <v>February</v>
+      </c>
+      <c r="C12" s="88">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E12" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F12" s="83"/>
+      <c r="G12" s="82"/>
+      <c r="H12" s="82"/>
+      <c r="I12" s="82"/>
+      <c r="J12" s="82"/>
+      <c r="K12" s="90"/>
+      <c r="L12" s="82"/>
+    </row>
+    <row r="13" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B13" s="67" t="str">
+        <v>March</v>
+      </c>
+      <c r="C13" s="88">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E13" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F13" s="83"/>
+      <c r="G13" s="82"/>
+      <c r="H13" s="82"/>
+      <c r="I13" s="82"/>
+      <c r="J13" s="82"/>
+      <c r="K13" s="90"/>
+      <c r="L13" s="82"/>
+    </row>
+    <row r="14" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B14" s="67" t="str">
+        <v>April</v>
+      </c>
+      <c r="C14" s="88">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E14" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F14" s="83"/>
+      <c r="G14" s="82"/>
+      <c r="H14" s="82"/>
+      <c r="I14" s="82"/>
+      <c r="J14" s="82"/>
+      <c r="K14" s="90"/>
+      <c r="L14" s="82"/>
+    </row>
+    <row r="15" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B15" s="67" t="str">
+        <v>May</v>
+      </c>
+      <c r="C15" s="88">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E15" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F15" s="83"/>
+      <c r="G15" s="82"/>
+      <c r="H15" s="82"/>
+      <c r="I15" s="82"/>
+      <c r="J15" s="82"/>
+      <c r="K15" s="90"/>
+      <c r="L15" s="82"/>
+    </row>
+    <row r="16" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B16" s="67" t="str">
+        <v>June</v>
+      </c>
+      <c r="C16" s="88">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E16" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F16" s="83"/>
+      <c r="G16" s="82"/>
+      <c r="H16" s="82"/>
+      <c r="I16" s="82"/>
+      <c r="J16" s="82"/>
+      <c r="K16" s="90"/>
+      <c r="L16" s="82"/>
+    </row>
+    <row r="17" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B17" s="67" t="str">
+        <v>July</v>
+      </c>
+      <c r="C17" s="88">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E17" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F17" s="83"/>
+      <c r="G17" s="82"/>
+      <c r="H17" s="82"/>
+      <c r="I17" s="82"/>
+      <c r="J17" s="82"/>
+      <c r="K17" s="90"/>
+      <c r="L17" s="82"/>
+    </row>
+    <row r="18" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B18" s="67" t="str">
+        <v>August</v>
+      </c>
+      <c r="C18" s="88">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E18" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F18" s="83"/>
+      <c r="G18" s="82"/>
+      <c r="H18" s="82"/>
+      <c r="I18" s="82"/>
+      <c r="J18" s="82"/>
+      <c r="K18" s="90"/>
+      <c r="L18" s="82"/>
+    </row>
+    <row r="19" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B19" s="67" t="str">
+        <v>September</v>
+      </c>
+      <c r="C19" s="88">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E19" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F19" s="83"/>
+      <c r="G19" s="82"/>
+      <c r="H19" s="82"/>
+      <c r="I19" s="82"/>
+      <c r="J19" s="82"/>
+      <c r="K19" s="90"/>
+      <c r="L19" s="82"/>
+    </row>
+    <row r="20" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B20" s="67" t="str">
+        <v>October</v>
+      </c>
+      <c r="C20" s="88">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E20" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F20" s="83"/>
+      <c r="G20" s="82"/>
+      <c r="H20" s="82"/>
+      <c r="I20" s="82"/>
+      <c r="J20" s="82"/>
+      <c r="K20" s="90"/>
+      <c r="L20" s="82"/>
+    </row>
+    <row r="21" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B21" s="67" t="str">
+        <v>November</v>
+      </c>
+      <c r="C21" s="88">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E21" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F21" s="83"/>
+      <c r="G21" s="82"/>
+      <c r="H21" s="82"/>
+      <c r="I21" s="82"/>
+      <c r="J21" s="82"/>
+      <c r="K21" s="90"/>
+      <c r="L21" s="82"/>
+    </row>
+    <row r="22" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="B22" s="67" t="str">
+        <v>December</v>
+      </c>
+      <c r="C22" s="88">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E22" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F22" s="83"/>
+      <c r="G22" s="82"/>
+      <c r="H22" s="82"/>
+      <c r="I22" s="82"/>
+      <c r="J22" s="82"/>
+      <c r="K22" s="90"/>
+      <c r="L22" s="82"/>
+    </row>
+    <row r="23" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E23" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F23" s="83"/>
+      <c r="G23" s="82"/>
+      <c r="H23" s="82"/>
+      <c r="I23" s="82"/>
+      <c r="J23" s="82"/>
+      <c r="K23" s="90"/>
+      <c r="L23" s="82"/>
+    </row>
+    <row r="24" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E24" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F24" s="83"/>
+      <c r="G24" s="82"/>
+      <c r="H24" s="82"/>
+      <c r="I24" s="82"/>
+      <c r="J24" s="82"/>
+      <c r="K24" s="90"/>
+      <c r="L24" s="82"/>
+    </row>
+    <row r="25" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E25" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F25" s="83"/>
+      <c r="G25" s="82"/>
+      <c r="H25" s="82"/>
+      <c r="I25" s="82"/>
+      <c r="J25" s="82"/>
+      <c r="K25" s="90"/>
+      <c r="L25" s="82"/>
+    </row>
+    <row r="26" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E26" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F26" s="83"/>
+      <c r="G26" s="82"/>
+      <c r="H26" s="82"/>
+      <c r="I26" s="82"/>
+      <c r="J26" s="82"/>
+      <c r="K26" s="90"/>
+      <c r="L26" s="82"/>
+    </row>
+    <row r="27" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E27" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F27" s="83"/>
+      <c r="G27" s="82"/>
+      <c r="H27" s="82"/>
+      <c r="I27" s="82"/>
+      <c r="J27" s="82"/>
+      <c r="K27" s="90"/>
+      <c r="L27" s="82"/>
+    </row>
+    <row r="28" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E28" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F28" s="83"/>
+      <c r="G28" s="82"/>
+      <c r="H28" s="82"/>
+      <c r="I28" s="82"/>
+      <c r="J28" s="82"/>
+      <c r="K28" s="90"/>
+      <c r="L28" s="82"/>
+    </row>
+    <row r="29" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E29" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F29" s="83"/>
+      <c r="G29" s="82"/>
+      <c r="H29" s="82"/>
+      <c r="I29" s="82"/>
+      <c r="J29" s="82"/>
+      <c r="K29" s="90"/>
+      <c r="L29" s="82"/>
+    </row>
+    <row r="30" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E30" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F30" s="83"/>
+      <c r="G30" s="82"/>
+      <c r="H30" s="82"/>
+      <c r="I30" s="82"/>
+      <c r="J30" s="82"/>
+      <c r="K30" s="90"/>
+      <c r="L30" s="82"/>
+    </row>
+    <row r="31" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E31" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F31" s="83"/>
+      <c r="G31" s="82"/>
+      <c r="H31" s="82"/>
+      <c r="I31" s="82"/>
+      <c r="J31" s="82"/>
+      <c r="K31" s="90"/>
+      <c r="L31" s="82"/>
+    </row>
+    <row r="32" spans="2:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E32" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F32" s="83"/>
+      <c r="G32" s="82"/>
+      <c r="H32" s="82"/>
+      <c r="I32" s="82"/>
+      <c r="J32" s="82"/>
+      <c r="K32" s="90"/>
+      <c r="L32" s="82"/>
+    </row>
+    <row r="33" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E33" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F33" s="83"/>
+      <c r="G33" s="82"/>
+      <c r="H33" s="82"/>
+      <c r="I33" s="82"/>
+      <c r="J33" s="82"/>
+      <c r="K33" s="90"/>
+      <c r="L33" s="82"/>
+    </row>
+    <row r="34" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E34" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F34" s="83"/>
+      <c r="G34" s="82"/>
+      <c r="H34" s="82"/>
+      <c r="I34" s="82"/>
+      <c r="J34" s="82"/>
+      <c r="K34" s="90"/>
+      <c r="L34" s="82"/>
+    </row>
+    <row r="35" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E35" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F35" s="83"/>
+      <c r="G35" s="82"/>
+      <c r="H35" s="82"/>
+      <c r="I35" s="82"/>
+      <c r="J35" s="82"/>
+      <c r="K35" s="90"/>
+      <c r="L35" s="82"/>
+    </row>
+    <row r="36" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E36" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F36" s="83"/>
+      <c r="G36" s="82"/>
+      <c r="H36" s="82"/>
+      <c r="I36" s="82"/>
+      <c r="J36" s="82"/>
+      <c r="K36" s="90"/>
+      <c r="L36" s="82"/>
+    </row>
+    <row r="37" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E37" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F37" s="83"/>
+      <c r="G37" s="82"/>
+      <c r="H37" s="82"/>
+      <c r="I37" s="82"/>
+      <c r="J37" s="82"/>
+      <c r="K37" s="90"/>
+      <c r="L37" s="82"/>
+    </row>
+    <row r="38" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E38" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F38" s="83"/>
+      <c r="G38" s="82"/>
+      <c r="H38" s="82"/>
+      <c r="I38" s="82"/>
+      <c r="J38" s="82"/>
+      <c r="K38" s="90"/>
+      <c r="L38" s="82"/>
+    </row>
+    <row r="39" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E39" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F39" s="83"/>
+      <c r="G39" s="82"/>
+      <c r="H39" s="82"/>
+      <c r="I39" s="82"/>
+      <c r="J39" s="82"/>
+      <c r="K39" s="90"/>
+      <c r="L39" s="82"/>
+    </row>
+    <row r="40" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E40" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F40" s="83"/>
+      <c r="G40" s="82"/>
+      <c r="H40" s="82"/>
+      <c r="I40" s="82"/>
+      <c r="J40" s="82"/>
+      <c r="K40" s="90"/>
+      <c r="L40" s="82"/>
+    </row>
+    <row r="41" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E41" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F41" s="83"/>
+      <c r="G41" s="82"/>
+      <c r="H41" s="82"/>
+      <c r="I41" s="82"/>
+      <c r="J41" s="82"/>
+      <c r="K41" s="90"/>
+      <c r="L41" s="82"/>
+    </row>
+    <row r="42" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E42" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F42" s="83"/>
+      <c r="G42" s="82"/>
+      <c r="H42" s="82"/>
+      <c r="I42" s="82"/>
+      <c r="J42" s="82"/>
+      <c r="K42" s="90"/>
+      <c r="L42" s="82"/>
+    </row>
+    <row r="43" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E43" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F43" s="83"/>
+      <c r="G43" s="82"/>
+      <c r="H43" s="82"/>
+      <c r="I43" s="82"/>
+      <c r="J43" s="82"/>
+      <c r="K43" s="90"/>
+      <c r="L43" s="82"/>
+    </row>
+    <row r="44" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E44" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F44" s="83"/>
+      <c r="G44" s="82"/>
+      <c r="H44" s="82"/>
+      <c r="I44" s="82"/>
+      <c r="J44" s="82"/>
+      <c r="K44" s="90"/>
+      <c r="L44" s="82"/>
+    </row>
+    <row r="45" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E45" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F45" s="83"/>
+      <c r="G45" s="82"/>
+      <c r="H45" s="82"/>
+      <c r="I45" s="82"/>
+      <c r="J45" s="82"/>
+      <c r="K45" s="90"/>
+      <c r="L45" s="82"/>
+    </row>
+    <row r="46" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E46" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F46" s="83"/>
+      <c r="G46" s="82"/>
+      <c r="H46" s="82"/>
+      <c r="I46" s="82"/>
+      <c r="J46" s="82"/>
+      <c r="K46" s="90"/>
+      <c r="L46" s="82"/>
+    </row>
+    <row r="47" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E47" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F47" s="83"/>
+      <c r="G47" s="82"/>
+      <c r="H47" s="82"/>
+      <c r="I47" s="82"/>
+      <c r="J47" s="82"/>
+      <c r="K47" s="90"/>
+      <c r="L47" s="82"/>
+    </row>
+    <row r="48" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E48" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F48" s="83"/>
+      <c r="G48" s="82"/>
+      <c r="H48" s="82"/>
+      <c r="I48" s="82"/>
+      <c r="J48" s="82"/>
+      <c r="K48" s="90"/>
+      <c r="L48" s="82"/>
+    </row>
+    <row r="49" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E49" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F49" s="83"/>
+      <c r="G49" s="82"/>
+      <c r="H49" s="82"/>
+      <c r="I49" s="82"/>
+      <c r="J49" s="82"/>
+      <c r="K49" s="90"/>
+      <c r="L49" s="82"/>
+    </row>
+    <row r="50" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E50" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F50" s="83"/>
+      <c r="G50" s="82"/>
+      <c r="H50" s="82"/>
+      <c r="I50" s="82"/>
+      <c r="J50" s="82"/>
+      <c r="K50" s="90"/>
+      <c r="L50" s="82"/>
+    </row>
+    <row r="51" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E51" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F51" s="83"/>
+      <c r="G51" s="82"/>
+      <c r="H51" s="82"/>
+      <c r="I51" s="82"/>
+      <c r="J51" s="82"/>
+      <c r="K51" s="90"/>
+      <c r="L51" s="82"/>
+    </row>
+    <row r="52" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E52" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F52" s="83"/>
+      <c r="G52" s="82"/>
+      <c r="H52" s="82"/>
+      <c r="I52" s="82"/>
+      <c r="J52" s="82"/>
+      <c r="K52" s="90"/>
+      <c r="L52" s="82"/>
+    </row>
+    <row r="53" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E53" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F53" s="83"/>
+      <c r="G53" s="82"/>
+      <c r="H53" s="82"/>
+      <c r="I53" s="82"/>
+      <c r="J53" s="82"/>
+      <c r="K53" s="90"/>
+      <c r="L53" s="82"/>
+    </row>
+    <row r="54" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E54" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F54" s="83"/>
+      <c r="G54" s="82"/>
+      <c r="H54" s="82"/>
+      <c r="I54" s="82"/>
+      <c r="J54" s="82"/>
+      <c r="K54" s="90"/>
+      <c r="L54" s="82"/>
+    </row>
+    <row r="55" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E55" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F55" s="83"/>
+      <c r="G55" s="82"/>
+      <c r="H55" s="82"/>
+      <c r="I55" s="82"/>
+      <c r="J55" s="82"/>
+      <c r="K55" s="90"/>
+      <c r="L55" s="82"/>
+    </row>
+    <row r="56" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E56" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F56" s="83"/>
+      <c r="G56" s="82"/>
+      <c r="H56" s="82"/>
+      <c r="I56" s="82"/>
+      <c r="J56" s="82"/>
+      <c r="K56" s="90"/>
+      <c r="L56" s="82"/>
+    </row>
+    <row r="57" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E57" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F57" s="83"/>
+      <c r="G57" s="82"/>
+      <c r="H57" s="82"/>
+      <c r="I57" s="82"/>
+      <c r="J57" s="82"/>
+      <c r="K57" s="90"/>
+      <c r="L57" s="82"/>
+    </row>
+    <row r="58" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E58" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F58" s="83"/>
+      <c r="G58" s="82"/>
+      <c r="H58" s="82"/>
+      <c r="I58" s="82"/>
+      <c r="J58" s="82"/>
+      <c r="K58" s="90"/>
+      <c r="L58" s="82"/>
+    </row>
+    <row r="59" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E59" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F59" s="83"/>
+      <c r="G59" s="82"/>
+      <c r="H59" s="82"/>
+      <c r="I59" s="82"/>
+      <c r="J59" s="82"/>
+      <c r="K59" s="90"/>
+      <c r="L59" s="82"/>
+    </row>
+    <row r="60" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E60" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F60" s="83"/>
+      <c r="G60" s="82"/>
+      <c r="H60" s="82"/>
+      <c r="I60" s="82"/>
+      <c r="J60" s="82"/>
+      <c r="K60" s="90"/>
+      <c r="L60" s="82"/>
+    </row>
+    <row r="61" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E61" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F61" s="83"/>
+      <c r="G61" s="82"/>
+      <c r="H61" s="82"/>
+      <c r="I61" s="82"/>
+      <c r="J61" s="82"/>
+      <c r="K61" s="90"/>
+      <c r="L61" s="82"/>
+    </row>
+    <row r="62" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E62" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F62" s="83"/>
+      <c r="G62" s="82"/>
+      <c r="H62" s="82"/>
+      <c r="I62" s="82"/>
+      <c r="J62" s="82"/>
+      <c r="K62" s="90"/>
+      <c r="L62" s="82"/>
+    </row>
+    <row r="63" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E63" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F63" s="83"/>
+      <c r="G63" s="82"/>
+      <c r="H63" s="82"/>
+      <c r="I63" s="82"/>
+      <c r="J63" s="82"/>
+      <c r="K63" s="90"/>
+      <c r="L63" s="82"/>
+    </row>
+    <row r="64" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E64" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F64" s="83"/>
+      <c r="G64" s="82"/>
+      <c r="H64" s="82"/>
+      <c r="I64" s="82"/>
+      <c r="J64" s="82"/>
+      <c r="K64" s="90"/>
+      <c r="L64" s="82"/>
+    </row>
+    <row r="65" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E65" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F65" s="83"/>
+      <c r="G65" s="82"/>
+      <c r="H65" s="82"/>
+      <c r="I65" s="82"/>
+      <c r="J65" s="82"/>
+      <c r="K65" s="90"/>
+      <c r="L65" s="82"/>
+    </row>
+    <row r="66" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E66" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F66" s="83"/>
+      <c r="G66" s="82"/>
+      <c r="H66" s="82"/>
+      <c r="I66" s="82"/>
+      <c r="J66" s="82"/>
+      <c r="K66" s="90"/>
+      <c r="L66" s="82"/>
+    </row>
+    <row r="67" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E67" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F67" s="83"/>
+      <c r="G67" s="82"/>
+      <c r="H67" s="82"/>
+      <c r="I67" s="82"/>
+      <c r="J67" s="82"/>
+      <c r="K67" s="90"/>
+      <c r="L67" s="82"/>
+    </row>
+    <row r="68" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E68" s="82" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F68" s="83"/>
+      <c r="G68" s="82"/>
+      <c r="H68" s="82"/>
+      <c r="I68" s="82"/>
+      <c r="J68" s="82"/>
+      <c r="K68" s="90"/>
+      <c r="L68" s="82"/>
+    </row>
+    <row r="69" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E69" s="82" t="str">
+        <f t="shared" ref="E69:E132" si="2">IF(ISBLANK(F69),"",F69-F68)</f>
+        <v/>
+      </c>
+      <c r="F69" s="83"/>
+      <c r="G69" s="82"/>
+      <c r="H69" s="82"/>
+      <c r="I69" s="82"/>
+      <c r="J69" s="82"/>
+      <c r="K69" s="90"/>
+      <c r="L69" s="82"/>
+    </row>
+    <row r="70" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E70" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F70" s="83"/>
+      <c r="G70" s="82"/>
+      <c r="H70" s="82"/>
+      <c r="I70" s="82"/>
+      <c r="J70" s="82"/>
+      <c r="K70" s="90"/>
+      <c r="L70" s="82"/>
+    </row>
+    <row r="71" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E71" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F71" s="83"/>
+      <c r="G71" s="82"/>
+      <c r="H71" s="82"/>
+      <c r="I71" s="82"/>
+      <c r="J71" s="82"/>
+      <c r="K71" s="90"/>
+      <c r="L71" s="82"/>
+    </row>
+    <row r="72" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E72" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F72" s="83"/>
+      <c r="G72" s="82"/>
+      <c r="H72" s="82"/>
+      <c r="I72" s="82"/>
+      <c r="J72" s="82"/>
+      <c r="K72" s="90"/>
+      <c r="L72" s="82"/>
+    </row>
+    <row r="73" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E73" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F73" s="83"/>
+      <c r="G73" s="82"/>
+      <c r="H73" s="82"/>
+      <c r="I73" s="82"/>
+      <c r="J73" s="82"/>
+      <c r="K73" s="90"/>
+      <c r="L73" s="82"/>
+    </row>
+    <row r="74" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E74" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F74" s="83"/>
+      <c r="G74" s="82"/>
+      <c r="H74" s="82"/>
+      <c r="I74" s="82"/>
+      <c r="J74" s="82"/>
+      <c r="K74" s="90"/>
+      <c r="L74" s="82"/>
+    </row>
+    <row r="75" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E75" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F75" s="83"/>
+      <c r="G75" s="82"/>
+      <c r="H75" s="82"/>
+      <c r="I75" s="82"/>
+      <c r="J75" s="82"/>
+      <c r="K75" s="90"/>
+      <c r="L75" s="82"/>
+    </row>
+    <row r="76" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E76" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F76" s="83"/>
+      <c r="G76" s="82"/>
+      <c r="H76" s="82"/>
+      <c r="I76" s="82"/>
+      <c r="J76" s="82"/>
+      <c r="K76" s="90"/>
+      <c r="L76" s="82"/>
+    </row>
+    <row r="77" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E77" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F77" s="83"/>
+      <c r="G77" s="82"/>
+      <c r="H77" s="82"/>
+      <c r="I77" s="82"/>
+      <c r="J77" s="82"/>
+      <c r="K77" s="90"/>
+      <c r="L77" s="82"/>
+    </row>
+    <row r="78" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E78" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F78" s="83"/>
+      <c r="G78" s="82"/>
+      <c r="H78" s="82"/>
+      <c r="I78" s="82"/>
+      <c r="J78" s="82"/>
+      <c r="K78" s="90"/>
+      <c r="L78" s="82"/>
+    </row>
+    <row r="79" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E79" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F79" s="83"/>
+      <c r="G79" s="82"/>
+      <c r="H79" s="82"/>
+      <c r="I79" s="82"/>
+      <c r="J79" s="82"/>
+      <c r="K79" s="90"/>
+      <c r="L79" s="82"/>
+    </row>
+    <row r="80" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E80" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F80" s="83"/>
+      <c r="G80" s="82"/>
+      <c r="H80" s="82"/>
+      <c r="I80" s="82"/>
+      <c r="J80" s="82"/>
+      <c r="K80" s="90"/>
+      <c r="L80" s="82"/>
+    </row>
+    <row r="81" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E81" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F81" s="83"/>
+      <c r="G81" s="82"/>
+      <c r="H81" s="82"/>
+      <c r="I81" s="82"/>
+      <c r="J81" s="82"/>
+      <c r="K81" s="90"/>
+      <c r="L81" s="82"/>
+    </row>
+    <row r="82" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E82" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F82" s="83"/>
+      <c r="G82" s="82"/>
+      <c r="H82" s="82"/>
+      <c r="I82" s="82"/>
+      <c r="J82" s="82"/>
+      <c r="K82" s="90"/>
+      <c r="L82" s="82"/>
+    </row>
+    <row r="83" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E83" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F83" s="83"/>
+      <c r="G83" s="82"/>
+      <c r="H83" s="82"/>
+      <c r="I83" s="82"/>
+      <c r="J83" s="82"/>
+      <c r="K83" s="90"/>
+      <c r="L83" s="82"/>
+    </row>
+    <row r="84" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E84" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F84" s="83"/>
+      <c r="G84" s="82"/>
+      <c r="H84" s="82"/>
+      <c r="I84" s="82"/>
+      <c r="J84" s="82"/>
+      <c r="K84" s="90"/>
+      <c r="L84" s="82"/>
+    </row>
+    <row r="85" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E85" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F85" s="83"/>
+      <c r="G85" s="82"/>
+      <c r="H85" s="82"/>
+      <c r="I85" s="82"/>
+      <c r="J85" s="82"/>
+      <c r="K85" s="90"/>
+      <c r="L85" s="82"/>
+    </row>
+    <row r="86" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E86" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F86" s="83"/>
+      <c r="G86" s="82"/>
+      <c r="H86" s="82"/>
+      <c r="I86" s="82"/>
+      <c r="J86" s="82"/>
+      <c r="K86" s="90"/>
+      <c r="L86" s="82"/>
+    </row>
+    <row r="87" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E87" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F87" s="83"/>
+      <c r="G87" s="82"/>
+      <c r="H87" s="82"/>
+      <c r="I87" s="82"/>
+      <c r="J87" s="82"/>
+      <c r="K87" s="90"/>
+      <c r="L87" s="82"/>
+    </row>
+    <row r="88" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E88" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F88" s="83"/>
+      <c r="G88" s="82"/>
+      <c r="H88" s="82"/>
+      <c r="I88" s="82"/>
+      <c r="J88" s="82"/>
+      <c r="K88" s="90"/>
+      <c r="L88" s="82"/>
+    </row>
+    <row r="89" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E89" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F89" s="83"/>
+      <c r="G89" s="82"/>
+      <c r="H89" s="82"/>
+      <c r="I89" s="82"/>
+      <c r="J89" s="82"/>
+      <c r="K89" s="90"/>
+      <c r="L89" s="82"/>
+    </row>
+    <row r="90" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E90" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F90" s="83"/>
+      <c r="G90" s="82"/>
+      <c r="H90" s="82"/>
+      <c r="I90" s="82"/>
+      <c r="J90" s="82"/>
+      <c r="K90" s="90"/>
+      <c r="L90" s="82"/>
+    </row>
+    <row r="91" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E91" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F91" s="83"/>
+      <c r="G91" s="82"/>
+      <c r="H91" s="82"/>
+      <c r="I91" s="82"/>
+      <c r="J91" s="82"/>
+      <c r="K91" s="90"/>
+      <c r="L91" s="82"/>
+    </row>
+    <row r="92" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E92" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F92" s="83"/>
+      <c r="G92" s="82"/>
+      <c r="H92" s="82"/>
+      <c r="I92" s="82"/>
+      <c r="J92" s="82"/>
+      <c r="K92" s="90"/>
+      <c r="L92" s="82"/>
+    </row>
+    <row r="93" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E93" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F93" s="83"/>
+      <c r="G93" s="82"/>
+      <c r="H93" s="82"/>
+      <c r="I93" s="82"/>
+      <c r="J93" s="82"/>
+      <c r="K93" s="90"/>
+      <c r="L93" s="82"/>
+    </row>
+    <row r="94" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E94" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F94" s="83"/>
+      <c r="G94" s="82"/>
+      <c r="H94" s="82"/>
+      <c r="I94" s="82"/>
+      <c r="J94" s="82"/>
+      <c r="K94" s="90"/>
+      <c r="L94" s="82"/>
+    </row>
+    <row r="95" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E95" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F95" s="83"/>
+      <c r="G95" s="82"/>
+      <c r="H95" s="82"/>
+      <c r="I95" s="82"/>
+      <c r="J95" s="82"/>
+      <c r="K95" s="90"/>
+      <c r="L95" s="82"/>
+    </row>
+    <row r="96" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E96" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F96" s="83"/>
+      <c r="G96" s="82"/>
+      <c r="H96" s="82"/>
+      <c r="I96" s="82"/>
+      <c r="J96" s="82"/>
+      <c r="K96" s="90"/>
+      <c r="L96" s="82"/>
+    </row>
+    <row r="97" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E97" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F97" s="83"/>
+      <c r="G97" s="82"/>
+      <c r="H97" s="82"/>
+      <c r="I97" s="82"/>
+      <c r="J97" s="82"/>
+      <c r="K97" s="90"/>
+      <c r="L97" s="82"/>
+    </row>
+    <row r="98" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E98" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F98" s="83"/>
+      <c r="G98" s="82"/>
+      <c r="H98" s="82"/>
+      <c r="I98" s="82"/>
+      <c r="J98" s="82"/>
+      <c r="K98" s="90"/>
+      <c r="L98" s="82"/>
+    </row>
+    <row r="99" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E99" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F99" s="83"/>
+      <c r="G99" s="82"/>
+      <c r="H99" s="82"/>
+      <c r="I99" s="82"/>
+      <c r="J99" s="82"/>
+      <c r="K99" s="90"/>
+      <c r="L99" s="82"/>
+    </row>
+    <row r="100" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E100" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F100" s="83"/>
+      <c r="G100" s="82"/>
+      <c r="H100" s="82"/>
+      <c r="I100" s="82"/>
+      <c r="J100" s="82"/>
+      <c r="K100" s="90"/>
+      <c r="L100" s="82"/>
+    </row>
+    <row r="101" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E101" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F101" s="83"/>
+      <c r="G101" s="82"/>
+      <c r="H101" s="82"/>
+      <c r="I101" s="82"/>
+      <c r="J101" s="82"/>
+      <c r="K101" s="90"/>
+      <c r="L101" s="82"/>
+    </row>
+    <row r="102" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E102" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F102" s="83"/>
+      <c r="G102" s="82"/>
+      <c r="H102" s="82"/>
+      <c r="I102" s="82"/>
+      <c r="J102" s="82"/>
+      <c r="K102" s="90"/>
+      <c r="L102" s="82"/>
+    </row>
+    <row r="103" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E103" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F103" s="83"/>
+      <c r="G103" s="82"/>
+      <c r="H103" s="82"/>
+      <c r="I103" s="82"/>
+      <c r="J103" s="82"/>
+      <c r="K103" s="90"/>
+      <c r="L103" s="82"/>
+    </row>
+    <row r="104" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E104" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F104" s="83"/>
+      <c r="G104" s="82"/>
+      <c r="H104" s="82"/>
+      <c r="I104" s="82"/>
+      <c r="J104" s="82"/>
+      <c r="K104" s="90"/>
+      <c r="L104" s="82"/>
+    </row>
+    <row r="105" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E105" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F105" s="83"/>
+      <c r="G105" s="82"/>
+      <c r="H105" s="82"/>
+      <c r="I105" s="82"/>
+      <c r="J105" s="82"/>
+      <c r="K105" s="90"/>
+      <c r="L105" s="82"/>
+    </row>
+    <row r="106" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E106" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F106" s="83"/>
+      <c r="G106" s="82"/>
+      <c r="H106" s="82"/>
+      <c r="I106" s="82"/>
+      <c r="J106" s="82"/>
+      <c r="K106" s="90"/>
+      <c r="L106" s="82"/>
+    </row>
+    <row r="107" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E107" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F107" s="83"/>
+      <c r="G107" s="82"/>
+      <c r="H107" s="82"/>
+      <c r="I107" s="82"/>
+      <c r="J107" s="82"/>
+      <c r="K107" s="90"/>
+      <c r="L107" s="82"/>
+    </row>
+    <row r="108" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E108" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F108" s="83"/>
+      <c r="G108" s="82"/>
+      <c r="H108" s="82"/>
+      <c r="I108" s="82"/>
+      <c r="J108" s="82"/>
+      <c r="K108" s="90"/>
+      <c r="L108" s="82"/>
+    </row>
+    <row r="109" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E109" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F109" s="83"/>
+      <c r="G109" s="82"/>
+      <c r="H109" s="82"/>
+      <c r="I109" s="82"/>
+      <c r="J109" s="82"/>
+      <c r="K109" s="90"/>
+      <c r="L109" s="82"/>
+    </row>
+    <row r="110" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E110" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F110" s="83"/>
+      <c r="G110" s="82"/>
+      <c r="H110" s="82"/>
+      <c r="I110" s="82"/>
+      <c r="J110" s="82"/>
+      <c r="K110" s="90"/>
+      <c r="L110" s="82"/>
+    </row>
+    <row r="111" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E111" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F111" s="83"/>
+      <c r="G111" s="82"/>
+      <c r="H111" s="82"/>
+      <c r="I111" s="82"/>
+      <c r="J111" s="82"/>
+      <c r="K111" s="90"/>
+      <c r="L111" s="82"/>
+    </row>
+    <row r="112" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E112" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F112" s="83"/>
+      <c r="G112" s="82"/>
+      <c r="H112" s="82"/>
+      <c r="I112" s="82"/>
+      <c r="J112" s="82"/>
+      <c r="K112" s="90"/>
+      <c r="L112" s="82"/>
+    </row>
+    <row r="113" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E113" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F113" s="83"/>
+      <c r="G113" s="82"/>
+      <c r="H113" s="82"/>
+      <c r="I113" s="82"/>
+      <c r="J113" s="82"/>
+      <c r="K113" s="90"/>
+      <c r="L113" s="82"/>
+    </row>
+    <row r="114" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E114" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F114" s="83"/>
+      <c r="G114" s="82"/>
+      <c r="H114" s="82"/>
+      <c r="I114" s="82"/>
+      <c r="J114" s="82"/>
+      <c r="K114" s="90"/>
+      <c r="L114" s="82"/>
+    </row>
+    <row r="115" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E115" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F115" s="83"/>
+      <c r="G115" s="82"/>
+      <c r="H115" s="82"/>
+      <c r="I115" s="82"/>
+      <c r="J115" s="82"/>
+      <c r="K115" s="90"/>
+      <c r="L115" s="82"/>
+    </row>
+    <row r="116" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E116" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F116" s="83"/>
+      <c r="G116" s="82"/>
+      <c r="H116" s="82"/>
+      <c r="I116" s="82"/>
+      <c r="J116" s="82"/>
+      <c r="K116" s="90"/>
+      <c r="L116" s="82"/>
+    </row>
+    <row r="117" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E117" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F117" s="83"/>
+      <c r="G117" s="82"/>
+      <c r="H117" s="82"/>
+      <c r="I117" s="82"/>
+      <c r="J117" s="82"/>
+      <c r="K117" s="90"/>
+      <c r="L117" s="82"/>
+    </row>
+    <row r="118" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E118" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F118" s="83"/>
+      <c r="G118" s="82"/>
+      <c r="H118" s="82"/>
+      <c r="I118" s="82"/>
+      <c r="J118" s="82"/>
+      <c r="K118" s="90"/>
+      <c r="L118" s="82"/>
+    </row>
+    <row r="119" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E119" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F119" s="83"/>
+      <c r="G119" s="82"/>
+      <c r="H119" s="82"/>
+      <c r="I119" s="82"/>
+      <c r="J119" s="82"/>
+      <c r="K119" s="90"/>
+      <c r="L119" s="82"/>
+    </row>
+    <row r="120" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E120" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F120" s="83"/>
+      <c r="G120" s="82"/>
+      <c r="H120" s="82"/>
+      <c r="I120" s="82"/>
+      <c r="J120" s="82"/>
+      <c r="K120" s="90"/>
+      <c r="L120" s="82"/>
+    </row>
+    <row r="121" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E121" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F121" s="83"/>
+      <c r="G121" s="82"/>
+      <c r="H121" s="82"/>
+      <c r="I121" s="82"/>
+      <c r="J121" s="82"/>
+      <c r="K121" s="90"/>
+      <c r="L121" s="82"/>
+    </row>
+    <row r="122" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E122" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F122" s="83"/>
+      <c r="G122" s="82"/>
+      <c r="H122" s="82"/>
+      <c r="I122" s="82"/>
+      <c r="J122" s="82"/>
+      <c r="K122" s="90"/>
+      <c r="L122" s="82"/>
+    </row>
+    <row r="123" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E123" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F123" s="83"/>
+      <c r="G123" s="82"/>
+      <c r="H123" s="82"/>
+      <c r="I123" s="82"/>
+      <c r="J123" s="82"/>
+      <c r="K123" s="90"/>
+      <c r="L123" s="82"/>
+    </row>
+    <row r="124" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E124" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F124" s="83"/>
+      <c r="G124" s="82"/>
+      <c r="H124" s="82"/>
+      <c r="I124" s="82"/>
+      <c r="J124" s="82"/>
+      <c r="K124" s="90"/>
+      <c r="L124" s="82"/>
+    </row>
+    <row r="125" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E125" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F125" s="83"/>
+      <c r="G125" s="82"/>
+      <c r="H125" s="82"/>
+      <c r="I125" s="82"/>
+      <c r="J125" s="82"/>
+      <c r="K125" s="90"/>
+      <c r="L125" s="82"/>
+    </row>
+    <row r="126" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E126" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F126" s="83"/>
+      <c r="G126" s="82"/>
+      <c r="H126" s="82"/>
+      <c r="I126" s="82"/>
+      <c r="J126" s="82"/>
+      <c r="K126" s="90"/>
+      <c r="L126" s="82"/>
+    </row>
+    <row r="127" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E127" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F127" s="83"/>
+      <c r="G127" s="82"/>
+      <c r="H127" s="82"/>
+      <c r="I127" s="82"/>
+      <c r="J127" s="82"/>
+      <c r="K127" s="90"/>
+      <c r="L127" s="82"/>
+    </row>
+    <row r="128" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E128" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F128" s="83"/>
+      <c r="G128" s="82"/>
+      <c r="H128" s="82"/>
+      <c r="I128" s="82"/>
+      <c r="J128" s="82"/>
+      <c r="K128" s="90"/>
+      <c r="L128" s="82"/>
+    </row>
+    <row r="129" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E129" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F129" s="83"/>
+      <c r="G129" s="82"/>
+      <c r="H129" s="82"/>
+      <c r="I129" s="82"/>
+      <c r="J129" s="82"/>
+      <c r="K129" s="90"/>
+      <c r="L129" s="82"/>
+    </row>
+    <row r="130" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E130" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F130" s="83"/>
+      <c r="G130" s="82"/>
+      <c r="H130" s="82"/>
+      <c r="I130" s="82"/>
+      <c r="J130" s="82"/>
+      <c r="K130" s="90"/>
+      <c r="L130" s="82"/>
+    </row>
+    <row r="131" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E131" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F131" s="83"/>
+      <c r="G131" s="82"/>
+      <c r="H131" s="82"/>
+      <c r="I131" s="82"/>
+      <c r="J131" s="82"/>
+      <c r="K131" s="90"/>
+      <c r="L131" s="82"/>
+    </row>
+    <row r="132" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E132" s="82" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F132" s="83"/>
+      <c r="G132" s="82"/>
+      <c r="H132" s="82"/>
+      <c r="I132" s="82"/>
+      <c r="J132" s="82"/>
+      <c r="K132" s="90"/>
+      <c r="L132" s="82"/>
+    </row>
+    <row r="133" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E133" s="82" t="str">
+        <f t="shared" ref="E133:E185" si="3">IF(ISBLANK(F133),"",F133-F132)</f>
+        <v/>
+      </c>
+      <c r="F133" s="83"/>
+      <c r="G133" s="82"/>
+      <c r="H133" s="82"/>
+      <c r="I133" s="82"/>
+      <c r="J133" s="82"/>
+      <c r="K133" s="90"/>
+      <c r="L133" s="82"/>
+    </row>
+    <row r="134" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E134" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F134" s="83"/>
+      <c r="G134" s="82"/>
+      <c r="H134" s="82"/>
+      <c r="I134" s="82"/>
+      <c r="J134" s="82"/>
+      <c r="K134" s="90"/>
+      <c r="L134" s="82"/>
+    </row>
+    <row r="135" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E135" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F135" s="83"/>
+      <c r="G135" s="82"/>
+      <c r="H135" s="82"/>
+      <c r="I135" s="82"/>
+      <c r="J135" s="82"/>
+      <c r="K135" s="90"/>
+      <c r="L135" s="82"/>
+    </row>
+    <row r="136" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E136" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F136" s="83"/>
+      <c r="G136" s="82"/>
+      <c r="H136" s="82"/>
+      <c r="I136" s="82"/>
+      <c r="J136" s="82"/>
+      <c r="K136" s="90"/>
+      <c r="L136" s="82"/>
+    </row>
+    <row r="137" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E137" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F137" s="83"/>
+      <c r="G137" s="82"/>
+      <c r="H137" s="82"/>
+      <c r="I137" s="82"/>
+      <c r="J137" s="82"/>
+      <c r="K137" s="90"/>
+      <c r="L137" s="82"/>
+    </row>
+    <row r="138" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E138" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F138" s="83"/>
+      <c r="G138" s="82"/>
+      <c r="H138" s="82"/>
+      <c r="I138" s="82"/>
+      <c r="J138" s="82"/>
+      <c r="K138" s="90"/>
+      <c r="L138" s="82"/>
+    </row>
+    <row r="139" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E139" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F139" s="83"/>
+      <c r="G139" s="82"/>
+      <c r="H139" s="82"/>
+      <c r="I139" s="82"/>
+      <c r="J139" s="82"/>
+      <c r="K139" s="90"/>
+      <c r="L139" s="82"/>
+    </row>
+    <row r="140" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E140" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F140" s="83"/>
+      <c r="G140" s="82"/>
+      <c r="H140" s="82"/>
+      <c r="I140" s="82"/>
+      <c r="J140" s="82"/>
+      <c r="K140" s="90"/>
+      <c r="L140" s="82"/>
+    </row>
+    <row r="141" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E141" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F141" s="83"/>
+      <c r="G141" s="82"/>
+      <c r="H141" s="82"/>
+      <c r="I141" s="82"/>
+      <c r="J141" s="82"/>
+      <c r="K141" s="90"/>
+      <c r="L141" s="82"/>
+    </row>
+    <row r="142" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E142" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F142" s="83"/>
+      <c r="G142" s="82"/>
+      <c r="H142" s="82"/>
+      <c r="I142" s="82"/>
+      <c r="J142" s="82"/>
+      <c r="K142" s="90"/>
+      <c r="L142" s="82"/>
+    </row>
+    <row r="143" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E143" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F143" s="83"/>
+      <c r="G143" s="82"/>
+      <c r="H143" s="82"/>
+      <c r="I143" s="82"/>
+      <c r="J143" s="82"/>
+      <c r="K143" s="90"/>
+      <c r="L143" s="82"/>
+    </row>
+    <row r="144" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E144" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F144" s="83"/>
+      <c r="G144" s="82"/>
+      <c r="H144" s="82"/>
+      <c r="I144" s="82"/>
+      <c r="J144" s="82"/>
+      <c r="K144" s="90"/>
+      <c r="L144" s="82"/>
+    </row>
+    <row r="145" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E145" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F145" s="83"/>
+      <c r="G145" s="82"/>
+      <c r="H145" s="82"/>
+      <c r="I145" s="82"/>
+      <c r="J145" s="82"/>
+      <c r="K145" s="90"/>
+      <c r="L145" s="82"/>
+    </row>
+    <row r="146" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E146" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F146" s="83"/>
+      <c r="G146" s="82"/>
+      <c r="H146" s="82"/>
+      <c r="I146" s="82"/>
+      <c r="J146" s="82"/>
+      <c r="K146" s="90"/>
+      <c r="L146" s="82"/>
+    </row>
+    <row r="147" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E147" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F147" s="83"/>
+      <c r="G147" s="82"/>
+      <c r="H147" s="82"/>
+      <c r="I147" s="82"/>
+      <c r="J147" s="82"/>
+      <c r="K147" s="90"/>
+      <c r="L147" s="82"/>
+    </row>
+    <row r="148" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E148" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F148" s="83"/>
+      <c r="G148" s="82"/>
+      <c r="H148" s="82"/>
+      <c r="I148" s="82"/>
+      <c r="J148" s="82"/>
+      <c r="K148" s="90"/>
+      <c r="L148" s="82"/>
+    </row>
+    <row r="149" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E149" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F149" s="83"/>
+      <c r="G149" s="82"/>
+      <c r="H149" s="82"/>
+      <c r="I149" s="82"/>
+      <c r="J149" s="82"/>
+      <c r="K149" s="90"/>
+      <c r="L149" s="82"/>
+    </row>
+    <row r="150" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E150" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F150" s="83"/>
+      <c r="G150" s="82"/>
+      <c r="H150" s="82"/>
+      <c r="I150" s="82"/>
+      <c r="J150" s="82"/>
+      <c r="K150" s="90"/>
+      <c r="L150" s="82"/>
+    </row>
+    <row r="151" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E151" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F151" s="83"/>
+      <c r="G151" s="82"/>
+      <c r="H151" s="82"/>
+      <c r="I151" s="82"/>
+      <c r="J151" s="82"/>
+      <c r="K151" s="90"/>
+      <c r="L151" s="82"/>
+    </row>
+    <row r="152" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E152" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F152" s="83"/>
+      <c r="G152" s="82"/>
+      <c r="H152" s="82"/>
+      <c r="I152" s="82"/>
+      <c r="J152" s="82"/>
+      <c r="K152" s="90"/>
+      <c r="L152" s="82"/>
+    </row>
+    <row r="153" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E153" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F153" s="83"/>
+      <c r="G153" s="82"/>
+      <c r="H153" s="82"/>
+      <c r="I153" s="82"/>
+      <c r="J153" s="82"/>
+      <c r="K153" s="90"/>
+      <c r="L153" s="82"/>
+    </row>
+    <row r="154" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E154" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F154" s="83"/>
+      <c r="G154" s="82"/>
+      <c r="H154" s="82"/>
+      <c r="I154" s="82"/>
+      <c r="J154" s="82"/>
+      <c r="K154" s="90"/>
+      <c r="L154" s="82"/>
+    </row>
+    <row r="155" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E155" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F155" s="83"/>
+      <c r="G155" s="82"/>
+      <c r="H155" s="82"/>
+      <c r="I155" s="82"/>
+      <c r="J155" s="82"/>
+      <c r="K155" s="90"/>
+      <c r="L155" s="82"/>
+    </row>
+    <row r="156" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E156" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F156" s="83"/>
+      <c r="G156" s="82"/>
+      <c r="H156" s="82"/>
+      <c r="I156" s="82"/>
+      <c r="J156" s="82"/>
+      <c r="K156" s="90"/>
+      <c r="L156" s="82"/>
+    </row>
+    <row r="157" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E157" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F157" s="83"/>
+      <c r="G157" s="82"/>
+      <c r="H157" s="82"/>
+      <c r="I157" s="82"/>
+      <c r="J157" s="82"/>
+      <c r="K157" s="90"/>
+      <c r="L157" s="82"/>
+    </row>
+    <row r="158" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E158" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F158" s="83"/>
+      <c r="G158" s="82"/>
+      <c r="H158" s="82"/>
+      <c r="I158" s="82"/>
+      <c r="J158" s="82"/>
+      <c r="K158" s="90"/>
+      <c r="L158" s="82"/>
+    </row>
+    <row r="159" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E159" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F159" s="83"/>
+      <c r="G159" s="82"/>
+      <c r="H159" s="82"/>
+      <c r="I159" s="82"/>
+      <c r="J159" s="82"/>
+      <c r="K159" s="90"/>
+      <c r="L159" s="82"/>
+    </row>
+    <row r="160" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E160" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F160" s="83"/>
+      <c r="G160" s="82"/>
+      <c r="H160" s="82"/>
+      <c r="I160" s="82"/>
+      <c r="J160" s="82"/>
+      <c r="K160" s="90"/>
+      <c r="L160" s="82"/>
+    </row>
+    <row r="161" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E161" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F161" s="83"/>
+      <c r="G161" s="82"/>
+      <c r="H161" s="82"/>
+      <c r="I161" s="82"/>
+      <c r="J161" s="82"/>
+      <c r="K161" s="90"/>
+      <c r="L161" s="82"/>
+    </row>
+    <row r="162" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E162" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F162" s="83"/>
+      <c r="G162" s="82"/>
+      <c r="H162" s="82"/>
+      <c r="I162" s="82"/>
+      <c r="J162" s="82"/>
+      <c r="K162" s="90"/>
+      <c r="L162" s="82"/>
+    </row>
+    <row r="163" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E163" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F163" s="83"/>
+      <c r="G163" s="82"/>
+      <c r="H163" s="82"/>
+      <c r="I163" s="82"/>
+      <c r="J163" s="82"/>
+      <c r="K163" s="90"/>
+      <c r="L163" s="82"/>
+    </row>
+    <row r="164" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E164" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F164" s="83"/>
+      <c r="G164" s="82"/>
+      <c r="H164" s="82"/>
+      <c r="I164" s="82"/>
+      <c r="J164" s="82"/>
+      <c r="K164" s="90"/>
+      <c r="L164" s="82"/>
+    </row>
+    <row r="165" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E165" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F165" s="83"/>
+      <c r="G165" s="82"/>
+      <c r="H165" s="82"/>
+      <c r="I165" s="82"/>
+      <c r="J165" s="82"/>
+      <c r="K165" s="90"/>
+      <c r="L165" s="82"/>
+    </row>
+    <row r="166" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E166" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F166" s="83"/>
+      <c r="G166" s="82"/>
+      <c r="H166" s="82"/>
+      <c r="I166" s="82"/>
+      <c r="J166" s="82"/>
+      <c r="K166" s="90"/>
+      <c r="L166" s="82"/>
+    </row>
+    <row r="167" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E167" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F167" s="83"/>
+      <c r="G167" s="82"/>
+      <c r="H167" s="82"/>
+      <c r="I167" s="82"/>
+      <c r="J167" s="82"/>
+      <c r="K167" s="90"/>
+      <c r="L167" s="82"/>
+    </row>
+    <row r="168" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E168" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F168" s="83"/>
+      <c r="G168" s="82"/>
+      <c r="H168" s="82"/>
+      <c r="I168" s="82"/>
+      <c r="J168" s="82"/>
+      <c r="K168" s="90"/>
+      <c r="L168" s="82"/>
+    </row>
+    <row r="169" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E169" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F169" s="83"/>
+      <c r="G169" s="82"/>
+      <c r="H169" s="82"/>
+      <c r="I169" s="82"/>
+      <c r="J169" s="82"/>
+      <c r="K169" s="90"/>
+      <c r="L169" s="82"/>
+    </row>
+    <row r="170" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E170" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F170" s="83"/>
+      <c r="G170" s="82"/>
+      <c r="H170" s="82"/>
+      <c r="I170" s="82"/>
+      <c r="J170" s="82"/>
+      <c r="K170" s="90"/>
+      <c r="L170" s="82"/>
+    </row>
+    <row r="171" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E171" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F171" s="83"/>
+      <c r="G171" s="82"/>
+      <c r="H171" s="82"/>
+      <c r="I171" s="82"/>
+      <c r="J171" s="82"/>
+      <c r="K171" s="90"/>
+      <c r="L171" s="82"/>
+    </row>
+    <row r="172" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E172" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F172" s="83"/>
+      <c r="G172" s="82"/>
+      <c r="H172" s="82"/>
+      <c r="I172" s="82"/>
+      <c r="J172" s="82"/>
+      <c r="K172" s="90"/>
+      <c r="L172" s="82"/>
+    </row>
+    <row r="173" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E173" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F173" s="83"/>
+      <c r="G173" s="82"/>
+      <c r="H173" s="82"/>
+      <c r="I173" s="82"/>
+      <c r="J173" s="82"/>
+      <c r="K173" s="90"/>
+      <c r="L173" s="82"/>
+    </row>
+    <row r="174" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E174" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F174" s="83"/>
+      <c r="G174" s="82"/>
+      <c r="H174" s="82"/>
+      <c r="I174" s="82"/>
+      <c r="J174" s="82"/>
+      <c r="K174" s="90"/>
+      <c r="L174" s="82"/>
+    </row>
+    <row r="175" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E175" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F175" s="83"/>
+      <c r="G175" s="82"/>
+      <c r="H175" s="82"/>
+      <c r="I175" s="82"/>
+      <c r="J175" s="82"/>
+      <c r="K175" s="90"/>
+      <c r="L175" s="82"/>
+    </row>
+    <row r="176" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E176" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F176" s="83"/>
+      <c r="G176" s="82"/>
+      <c r="H176" s="82"/>
+      <c r="I176" s="82"/>
+      <c r="J176" s="82"/>
+      <c r="K176" s="90"/>
+      <c r="L176" s="82"/>
+    </row>
+    <row r="177" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E177" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F177" s="83"/>
+      <c r="G177" s="82"/>
+      <c r="H177" s="82"/>
+      <c r="I177" s="82"/>
+      <c r="J177" s="82"/>
+      <c r="K177" s="90"/>
+      <c r="L177" s="82"/>
+    </row>
+    <row r="178" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E178" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F178" s="83"/>
+      <c r="G178" s="82"/>
+      <c r="H178" s="82"/>
+      <c r="I178" s="82"/>
+      <c r="J178" s="82"/>
+      <c r="K178" s="90"/>
+      <c r="L178" s="82"/>
+    </row>
+    <row r="179" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E179" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F179" s="83"/>
+      <c r="G179" s="82"/>
+      <c r="H179" s="82"/>
+      <c r="I179" s="82"/>
+      <c r="J179" s="82"/>
+      <c r="K179" s="90"/>
+      <c r="L179" s="82"/>
+    </row>
+    <row r="180" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E180" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F180" s="83"/>
+      <c r="G180" s="82"/>
+      <c r="H180" s="82"/>
+      <c r="I180" s="82"/>
+      <c r="J180" s="82"/>
+      <c r="K180" s="90"/>
+      <c r="L180" s="82"/>
+    </row>
+    <row r="181" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E181" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F181" s="83"/>
+      <c r="G181" s="82"/>
+      <c r="H181" s="82"/>
+      <c r="I181" s="82"/>
+      <c r="J181" s="82"/>
+      <c r="K181" s="90"/>
+      <c r="L181" s="82"/>
+    </row>
+    <row r="182" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E182" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F182" s="83"/>
+      <c r="G182" s="82"/>
+      <c r="H182" s="82"/>
+      <c r="I182" s="82"/>
+      <c r="J182" s="82"/>
+      <c r="K182" s="90"/>
+      <c r="L182" s="82"/>
+    </row>
+    <row r="183" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E183" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F183" s="83"/>
+      <c r="G183" s="82"/>
+      <c r="H183" s="82"/>
+      <c r="I183" s="82"/>
+      <c r="J183" s="82"/>
+      <c r="K183" s="90"/>
+      <c r="L183" s="82"/>
+    </row>
+    <row r="184" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E184" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F184" s="83"/>
+      <c r="G184" s="82"/>
+      <c r="H184" s="82"/>
+      <c r="I184" s="82"/>
+      <c r="J184" s="82"/>
+      <c r="K184" s="90"/>
+      <c r="L184" s="82"/>
+    </row>
+    <row r="185" spans="5:12" ht="15" x14ac:dyDescent="0.3">
+      <c r="E185" s="82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F185" s="83"/>
+      <c r="G185" s="82"/>
+      <c r="H185" s="82"/>
+      <c r="I185" s="82"/>
+      <c r="J185" s="82"/>
+      <c r="K185" s="90"/>
+      <c r="L185" s="82"/>
+    </row>
+    <row r="201" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B201" s="85">
+        <f>IF(ISBLANK(#REF!),"",C201-F185)</f>
+        <v>0</v>
+      </c>
+      <c r="C201" s="86"/>
+      <c r="D201" s="85"/>
+      <c r="E201" s="85"/>
+      <c r="F201" s="85"/>
+      <c r="G201" s="85"/>
+      <c r="H201" s="87"/>
+      <c r="I201" s="85"/>
+    </row>
+    <row r="202" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B202" s="85">
+        <f>IF(ISBLANK(#REF!),"",C202-C201)</f>
+        <v>0</v>
+      </c>
+      <c r="C202" s="86"/>
+      <c r="D202" s="85"/>
+      <c r="E202" s="85"/>
+      <c r="F202" s="85"/>
+      <c r="G202" s="85"/>
+      <c r="H202" s="87"/>
+      <c r="I202" s="85"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2" xr:uid="{EB042F53-BF78-4C94-A739-939262B37E1C}">
+      <formula1>INDIRECT("Tabela1[Description]")</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAD330F4-3FAE-447F-BF05-82EFBCBD7BD0}">
   <sheetPr codeName="Planilha6">
     <tabColor theme="1"/>
@@ -13077,15 +15732,15 @@
       <c r="I2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="79" t="s">
+      <c r="K2" s="78" t="s">
         <v>37</v>
       </c>
-      <c r="L2" s="80"/>
+      <c r="L2" s="79"/>
       <c r="M2" s="24"/>
-      <c r="N2" s="79" t="s">
+      <c r="N2" s="78" t="s">
         <v>43</v>
       </c>
-      <c r="O2" s="80"/>
+      <c r="O2" s="79"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="str" cm="1">

</xml_diff>